<commit_message>
docs: add more verified QML literature
</commit_message>
<xml_diff>
--- a/metadata/QML.xlsx
+++ b/metadata/QML.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7b2b7ba1cba44746"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rf3bd9b33c24e40fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -672,19 +672,19 @@
     </x:row>
     <x:row r="8" ht="15.75">
       <x:c r="A8" s="2" t="str">
-        <x:v>A Survey of Quantum Machine Learning: Foundations, Algorithms, Frameworks, Data and Applications</x:v>
+        <x:v>Noisy quantum learning theory</x:v>
       </x:c>
       <x:c r="B8" s="2" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
-        <x:v>ACM Computing Surveys</x:v>
+        <x:v>Nature Communications</x:v>
       </x:c>
       <x:c r="D8" s="2" t="str">
-        <x:v>Francesc Rodríguez-Díaz; David Gutiérrez-Avilés; Alicia Troncoso; Francisco Martínez-Álvarez</x:v>
+        <x:v>Jordan Cotler; Weiyuan Gong; Ishaan Kannan</x:v>
       </x:c>
       <x:c r="E8" s="2" t="str">
-        <x:v>https://doi.org/10.1145/3764582</x:v>
+        <x:v>https://doi.org/10.1038/s41467-026-73693-x</x:v>
       </x:c>
       <x:c r="F8" s="2" t="str">
         <x:v>QML</x:v>
@@ -692,19 +692,19 @@
     </x:row>
     <x:row r="9" ht="15.75">
       <x:c r="A9" s="2" t="str">
-        <x:v>Systematic literature review: Quantum machine learning and its applications</x:v>
+        <x:v>Quantum feature-map learning with reduced resource overhead</x:v>
       </x:c>
       <x:c r="B9" s="2" t="n">
-        <x:v>2024</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>Computer Science Review</x:v>
+        <x:v>Physical Review Research</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
-        <x:v>Peral-García, David, Juan Cruz-Benito, and Francisco José García-Peñalvo.</x:v>
+        <x:v>Jonas Jäger; Philipp Elsässer; Elham Torabian</x:v>
       </x:c>
       <x:c r="E9" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/pii/S1574013724000030</x:v>
+        <x:v>https://doi.org/10.1103/v29j-rh32</x:v>
       </x:c>
       <x:c r="F9" s="2" t="str">
         <x:v>QML</x:v>
@@ -712,182 +712,182 @@
     </x:row>
     <x:row r="10" ht="15.75">
       <x:c r="A10" s="2" t="str">
+        <x:v>Entanglement and classical simulability in quantum extreme-learning machines</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>Physical Review Applied</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="str">
+        <x:v>A. De Lorenzis; M. P. Casado; N. Lo Gullo; T. Lux; F. Plastina et al.</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="str">
+        <x:v>https://doi.org/10.1103/891x-ltcy</x:v>
+      </x:c>
+      <x:c r="F10" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15.75">
+      <x:c r="A11" s="2" t="str">
+        <x:v>A regularization method for quantum neural networks using data symmetry</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
+        <x:v>Discover Quantum Science</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="str">
+        <x:v>Hiroshi Ohno</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="str">
+        <x:v>https://doi.org/10.1007/s44464-026-00039-3</x:v>
+      </x:c>
+      <x:c r="F11" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15.75">
+      <x:c r="A12" s="2" t="str">
+        <x:v>A Survey of Quantum Machine Learning: Foundations, Algorithms, Frameworks, Data and Applications</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>ACM Computing Surveys</x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="str">
+        <x:v>Francesc Rodríguez-Díaz; David Gutiérrez-Avilés; Alicia Troncoso; Francisco Martínez-Álvarez</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="str">
+        <x:v>https://doi.org/10.1145/3764582</x:v>
+      </x:c>
+      <x:c r="F12" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15.75">
+      <x:c r="A13" s="2" t="str">
+        <x:v>Systematic literature review: Quantum machine learning and its applications</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>Computer Science Review</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="str">
+        <x:v>Peral-García, David, Juan Cruz-Benito, and Francisco José García-Peñalvo.</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/pii/S1574013724000030</x:v>
+      </x:c>
+      <x:c r="F13" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15.75">
+      <x:c r="A14" s="2" t="str">
         <x:v>Shadows of quantum machine learning
 </x:v>
       </x:c>
-      <x:c r="B10" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C10" s="2" t="str">
+      <x:c r="B14" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
         <x:v>Nature Communications</x:v>
       </x:c>
-      <x:c r="D10" s="2" t="str">
+      <x:c r="D14" s="2" t="str">
         <x:v>Jerbi, Sofiene, et al.</x:v>
       </x:c>
-      <x:c r="E10" s="2" t="str">
+      <x:c r="E14" s="2" t="str">
         <x:v>https://www.nature.com/articles/s41467-024-49877-8</x:v>
       </x:c>
-      <x:c r="F10" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="15.75">
-      <x:c r="A11" s="2" t="str">
+      <x:c r="F14" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15.75">
+      <x:c r="A15" s="2" t="str">
         <x:v>Quantum Machine Learning Revolution in Healthcare: A Systematic Review of Emerging Perspectives and Applications</x:v>
       </x:c>
-      <x:c r="B11" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C11" s="2" t="str">
+      <x:c r="B15" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
         <x:v>IEEE Access </x:v>
       </x:c>
-      <x:c r="D11" s="2" t="str">
+      <x:c r="D15" s="2" t="str">
         <x:v>Ullah, Ubaid, and Begonya Garcia-Zapirain.</x:v>
       </x:c>
-      <x:c r="E11" s="2" t="str">
+      <x:c r="E15" s="2" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10398184</x:v>
       </x:c>
-      <x:c r="F11" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15.75">
-      <x:c r="A12" s="2" t="str">
+      <x:c r="F15" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15.75">
+      <x:c r="A16" s="2" t="str">
         <x:v>Quantum machine learning for image classification</x:v>
       </x:c>
-      <x:c r="B12" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C12" s="2" t="str">
+      <x:c r="B16" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
         <x:v>Machine Learning: Science and Technology</x:v>
       </x:c>
-      <x:c r="D12" s="2" t="str">
+      <x:c r="D16" s="2" t="str">
         <x:v>Senokosov, Arsenii, et al.</x:v>
       </x:c>
-      <x:c r="E12" s="2" t="str">
+      <x:c r="E16" s="2" t="str">
         <x:v>https://iopscience.iop.org/article/10.1088/2632-2153/ad2aef/meta</x:v>
       </x:c>
-      <x:c r="F12" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="15.75">
-      <x:c r="A13" s="2" t="str">
+      <x:c r="F16" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15.75">
+      <x:c r="A17" s="2" t="str">
         <x:v>Quantum machine learning on near-term quantum devices: Current state of supervised and unsupervised techniques for real-world applications
 </x:v>
       </x:c>
-      <x:c r="B13" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C13" s="2" t="str">
+      <x:c r="B17" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
         <x:v>Physical Review Applied</x:v>
       </x:c>
-      <x:c r="D13" s="2" t="str">
+      <x:c r="D17" s="2" t="str">
         <x:v>Gujju, Yaswitha, Atsushi Matsuo, and Rudy Raymond.</x:v>
       </x:c>
-      <x:c r="E13" s="2" t="str">
+      <x:c r="E17" s="2" t="str">
         <x:v>https://journals.aps.org/prapplied/abstract/10.1103/PhysRevApplied.21.067001</x:v>
       </x:c>
-      <x:c r="F13" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="15.75">
-      <x:c r="A14" s="2" t="str">
+      <x:c r="F17" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15.75">
+      <x:c r="A18" s="2" t="str">
         <x:v>Better than classical? The subtle art of benchmarking quantum machine learning models
 </x:v>
       </x:c>
-      <x:c r="B14" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C14" s="2" t="str">
+      <x:c r="B18" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D14" s="2" t="str">
+      <x:c r="D18" s="2" t="str">
         <x:v>Bowles, Joseph, Shahnawaz Ahmed, and Maria Schuld.</x:v>
       </x:c>
-      <x:c r="E14" s="2" t="str">
+      <x:c r="E18" s="2" t="str">
         <x:v>https://arxiv.org/abs/2403.07059</x:v>
-      </x:c>
-      <x:c r="F14" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="15.75">
-      <x:c r="A15" s="2" t="str">
-        <x:v>Understanding quantum machine learning also requires rethinking generalization</x:v>
-      </x:c>
-      <x:c r="B15" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C15" s="2" t="str">
-        <x:v>Nature Communications </x:v>
-      </x:c>
-      <x:c r="D15" s="2" t="str">
-        <x:v>Gil-Fuster, Elies, Jens Eisert, and Carlos Bravo-Prieto.</x:v>
-      </x:c>
-      <x:c r="E15" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s41467-024-45882-z</x:v>
-      </x:c>
-      <x:c r="F15" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="15.75">
-      <x:c r="A16" s="2" t="str">
-        <x:v>Quantum machine learning for support vector machine classification</x:v>
-      </x:c>
-      <x:c r="B16" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C16" s="2" t="str">
-        <x:v>Evolutionary Intelligence </x:v>
-      </x:c>
-      <x:c r="D16" s="2" t="str">
-        <x:v>Kavitha, S. S., and Narasimha Kaulgud.</x:v>
-      </x:c>
-      <x:c r="E16" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s12065-022-00756-5</x:v>
-      </x:c>
-      <x:c r="F16" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="15.75">
-      <x:c r="A17" s="2" t="str">
-        <x:v>Provably Trainable Rotationally Equivariant Quantum Machine Learning</x:v>
-      </x:c>
-      <x:c r="B17" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C17" s="2" t="str">
-        <x:v>PRX Quantum </x:v>
-      </x:c>
-      <x:c r="D17" s="2" t="str">
-        <x:v>West, Maxwell T., et al.</x:v>
-      </x:c>
-      <x:c r="E17" s="2" t="str">
-        <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.5.030320</x:v>
-      </x:c>
-      <x:c r="F17" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="15.75">
-      <x:c r="A18" s="2" t="str">
-        <x:v>Quantum Machine Learning - Models and Algorithms: Studying quantum machine learning models and algorithms for leveraging quantum computing advantages in data analysis, pattern recognition, and optimization</x:v>
-      </x:c>
-      <x:c r="B18" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C18" s="2" t="str">
-        <x:v>Australian Journal of Machine Learning Research &amp; Applications</x:v>
-      </x:c>
-      <x:c r="D18" s="2" t="str">
-        <x:v>Abbas, Hassan.</x:v>
-      </x:c>
-      <x:c r="E18" s="2" t="str">
-        <x:v>https://sydneyacademics.com/index.php/ajmlra/article/view/68</x:v>
       </x:c>
       <x:c r="F18" s="2" t="str">
         <x:v>QML</x:v>
@@ -895,17 +895,19 @@
     </x:row>
     <x:row r="19" ht="15.75">
       <x:c r="A19" s="2" t="str">
-        <x:v>Quantum Machine Learning: Exploring the Potential of Quantum Computing forAI Applications</x:v>
+        <x:v>Understanding quantum machine learning also requires rethinking generalization</x:v>
       </x:c>
       <x:c r="B19" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C19" s="2"/>
+      <x:c r="C19" s="2" t="str">
+        <x:v>Nature Communications </x:v>
+      </x:c>
       <x:c r="D19" s="2" t="str">
-        <x:v>Potter, Kaledio, and Dylan Stilinski.</x:v>
+        <x:v>Gil-Fuster, Elies, Jens Eisert, and Carlos Bravo-Prieto.</x:v>
       </x:c>
       <x:c r="E19" s="2" t="str">
-        <x:v>-</x:v>
+        <x:v>https://www.nature.com/articles/s41467-024-45882-z</x:v>
       </x:c>
       <x:c r="F19" s="2" t="str">
         <x:v>QML</x:v>
@@ -913,19 +915,19 @@
     </x:row>
     <x:row r="20" ht="15.75">
       <x:c r="A20" s="2" t="str">
-        <x:v>Dynamical simulation via quantum machine learning with provable generalization</x:v>
+        <x:v>Quantum machine learning for support vector machine classification</x:v>
       </x:c>
       <x:c r="B20" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C20" s="2" t="str">
-        <x:v>Physical Review Research </x:v>
+        <x:v>Evolutionary Intelligence </x:v>
       </x:c>
       <x:c r="D20" s="2" t="str">
-        <x:v>Gibbs, Joe, et al.</x:v>
+        <x:v>Kavitha, S. S., and Narasimha Kaulgud.</x:v>
       </x:c>
       <x:c r="E20" s="2" t="str">
-        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.6.013241</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s12065-022-00756-5</x:v>
       </x:c>
       <x:c r="F20" s="2" t="str">
         <x:v>QML</x:v>
@@ -933,19 +935,19 @@
     </x:row>
     <x:row r="21" ht="15.75">
       <x:c r="A21" s="2" t="str">
-        <x:v>Symmetry Breaking in Geometric Quantum Machine Learning in the Presence of Noise</x:v>
+        <x:v>Provably Trainable Rotationally Equivariant Quantum Machine Learning</x:v>
       </x:c>
       <x:c r="B21" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C21" s="2" t="str">
-        <x:v>PRX Quantum</x:v>
+        <x:v>PRX Quantum </x:v>
       </x:c>
       <x:c r="D21" s="2" t="str">
-        <x:v>Tüysüz, Cenk, et al.</x:v>
+        <x:v>West, Maxwell T., et al.</x:v>
       </x:c>
       <x:c r="E21" s="2" t="str">
-        <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.5.030314</x:v>
+        <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.5.030320</x:v>
       </x:c>
       <x:c r="F21" s="2" t="str">
         <x:v>QML</x:v>
@@ -953,19 +955,19 @@
     </x:row>
     <x:row r="22" ht="15.75">
       <x:c r="A22" s="2" t="str">
-        <x:v>Generative Quantum Machine Learning via Denoising Diffusion Probabilistic Models</x:v>
+        <x:v>Quantum Machine Learning - Models and Algorithms: Studying quantum machine learning models and algorithms for leveraging quantum computing advantages in data analysis, pattern recognition, and optimization</x:v>
       </x:c>
       <x:c r="B22" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C22" s="2" t="str">
-        <x:v>Physical Review Letters </x:v>
+        <x:v>Australian Journal of Machine Learning Research &amp; Applications</x:v>
       </x:c>
       <x:c r="D22" s="2" t="str">
-        <x:v>Zhang, Bingzhi, et al.</x:v>
+        <x:v>Abbas, Hassan.</x:v>
       </x:c>
       <x:c r="E22" s="2" t="str">
-        <x:v>https://journals.aps.org/prl/abstract/10.1103/PhysRevLett.132.100602</x:v>
+        <x:v>https://sydneyacademics.com/index.php/ajmlra/article/view/68</x:v>
       </x:c>
       <x:c r="F22" s="2" t="str">
         <x:v>QML</x:v>
@@ -973,19 +975,17 @@
     </x:row>
     <x:row r="23" ht="15.75">
       <x:c r="A23" s="2" t="str">
-        <x:v>Applications of Quantum Machine Learning in Large-Scale E-commerce Recommendation Systems: Enhancing Efficiency and Accuracy</x:v>
+        <x:v>Quantum Machine Learning: Exploring the Potential of Quantum Computing forAI Applications</x:v>
       </x:c>
       <x:c r="B23" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C23" s="2" t="str">
-        <x:v>Journal of Industrial Engineering and Applied Science </x:v>
-      </x:c>
+      <x:c r="C23" s="2"/>
       <x:c r="D23" s="2" t="str">
-        <x:v>Shi, Jiatu, et al.</x:v>
+        <x:v>Potter, Kaledio, and Dylan Stilinski.</x:v>
       </x:c>
       <x:c r="E23" s="2" t="str">
-        <x:v>https://www.suaspress.org/ojs/index.php/JIEAS/article/view/v2n4a14</x:v>
+        <x:v>-</x:v>
       </x:c>
       <x:c r="F23" s="2" t="str">
         <x:v>QML</x:v>
@@ -993,19 +993,19 @@
     </x:row>
     <x:row r="24" ht="15.75">
       <x:c r="A24" s="2" t="str">
-        <x:v>An improved classical singular value transformation for quantum machine learning</x:v>
+        <x:v>Dynamical simulation via quantum machine learning with provable generalization</x:v>
       </x:c>
       <x:c r="B24" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C24" s="2" t="str">
-        <x:v>Annual ACM-SIAM Symposium on Discrete Algorithms (SODA)</x:v>
+        <x:v>Physical Review Research </x:v>
       </x:c>
       <x:c r="D24" s="2" t="str">
-        <x:v>Bakshi, Ainesh, and Ewin Tang.</x:v>
+        <x:v>Gibbs, Joe, et al.</x:v>
       </x:c>
       <x:c r="E24" s="2" t="str">
-        <x:v>https://epubs.siam.org/doi/abs/10.1137/1.9781611977912.86</x:v>
+        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.6.013241</x:v>
       </x:c>
       <x:c r="F24" s="2" t="str">
         <x:v>QML</x:v>
@@ -1013,19 +1013,19 @@
     </x:row>
     <x:row r="25" ht="15.75">
       <x:c r="A25" s="2" t="str">
-        <x:v>Blind Quantum Machine Learning with Quantum Bipartite Correlator</x:v>
+        <x:v>Symmetry Breaking in Geometric Quantum Machine Learning in the Presence of Noise</x:v>
       </x:c>
       <x:c r="B25" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C25" s="2" t="str">
-        <x:v>Physical Review Letters </x:v>
+        <x:v>PRX Quantum</x:v>
       </x:c>
       <x:c r="D25" s="2" t="str">
-        <x:v>Li, Changhao, et al.</x:v>
+        <x:v>Tüysüz, Cenk, et al.</x:v>
       </x:c>
       <x:c r="E25" s="2" t="str">
-        <x:v>https://journals.aps.org/prl/abstract/10.1103/PhysRevLett.133.120602</x:v>
+        <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.5.030314</x:v>
       </x:c>
       <x:c r="F25" s="2" t="str">
         <x:v>QML</x:v>
@@ -1033,19 +1033,19 @@
     </x:row>
     <x:row r="26" ht="15.75">
       <x:c r="A26" s="2" t="str">
-        <x:v>Quantum Machine Learning for Computational Methods in Engineering: A Systematic Review</x:v>
+        <x:v>Generative Quantum Machine Learning via Denoising Diffusion Probabilistic Models</x:v>
       </x:c>
       <x:c r="B26" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C26" s="2" t="str">
-        <x:v>Archives of Computational Methods in Engineering</x:v>
+        <x:v>Physical Review Letters </x:v>
       </x:c>
       <x:c r="D26" s="2" t="str">
-        <x:v>Sood, Sandeep Kumar, and Monika Agrewal.</x:v>
+        <x:v>Zhang, Bingzhi, et al.</x:v>
       </x:c>
       <x:c r="E26" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11831-023-10027-w</x:v>
+        <x:v>https://journals.aps.org/prl/abstract/10.1103/PhysRevLett.132.100602</x:v>
       </x:c>
       <x:c r="F26" s="2" t="str">
         <x:v>QML</x:v>
@@ -1053,19 +1053,19 @@
     </x:row>
     <x:row r="27" ht="15.75">
       <x:c r="A27" s="2" t="str">
-        <x:v>Overcoming the coherence time barrier in quantum machine learning on temporal data</x:v>
+        <x:v>Applications of Quantum Machine Learning in Large-Scale E-commerce Recommendation Systems: Enhancing Efficiency and Accuracy</x:v>
       </x:c>
       <x:c r="B27" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C27" s="2" t="str">
-        <x:v>Nature Communications </x:v>
+        <x:v>Journal of Industrial Engineering and Applied Science </x:v>
       </x:c>
       <x:c r="D27" s="2" t="str">
-        <x:v>Hu, Fangjun, et al.</x:v>
+        <x:v>Shi, Jiatu, et al.</x:v>
       </x:c>
       <x:c r="E27" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s41467-024-51162-7</x:v>
+        <x:v>https://www.suaspress.org/ojs/index.php/JIEAS/article/view/v2n4a14</x:v>
       </x:c>
       <x:c r="F27" s="2" t="str">
         <x:v>QML</x:v>
@@ -1073,428 +1073,428 @@
     </x:row>
     <x:row r="28" ht="15.75">
       <x:c r="A28" s="2" t="str">
+        <x:v>An improved classical singular value transformation for quantum machine learning</x:v>
+      </x:c>
+      <x:c r="B28" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
+        <x:v>Annual ACM-SIAM Symposium on Discrete Algorithms (SODA)</x:v>
+      </x:c>
+      <x:c r="D28" s="2" t="str">
+        <x:v>Bakshi, Ainesh, and Ewin Tang.</x:v>
+      </x:c>
+      <x:c r="E28" s="2" t="str">
+        <x:v>https://epubs.siam.org/doi/abs/10.1137/1.9781611977912.86</x:v>
+      </x:c>
+      <x:c r="F28" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="15.75">
+      <x:c r="A29" s="2" t="str">
+        <x:v>Blind Quantum Machine Learning with Quantum Bipartite Correlator</x:v>
+      </x:c>
+      <x:c r="B29" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C29" s="2" t="str">
+        <x:v>Physical Review Letters </x:v>
+      </x:c>
+      <x:c r="D29" s="2" t="str">
+        <x:v>Li, Changhao, et al.</x:v>
+      </x:c>
+      <x:c r="E29" s="2" t="str">
+        <x:v>https://journals.aps.org/prl/abstract/10.1103/PhysRevLett.133.120602</x:v>
+      </x:c>
+      <x:c r="F29" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="15.75">
+      <x:c r="A30" s="2" t="str">
+        <x:v>Quantum Machine Learning for Computational Methods in Engineering: A Systematic Review</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>Archives of Computational Methods in Engineering</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="str">
+        <x:v>Sood, Sandeep Kumar, and Monika Agrewal.</x:v>
+      </x:c>
+      <x:c r="E30" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s11831-023-10027-w</x:v>
+      </x:c>
+      <x:c r="F30" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="15.75">
+      <x:c r="A31" s="2" t="str">
+        <x:v>Overcoming the coherence time barrier in quantum machine learning on temporal data</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>Nature Communications </x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="str">
+        <x:v>Hu, Fangjun, et al.</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="str">
+        <x:v>https://www.nature.com/articles/s41467-024-51162-7</x:v>
+      </x:c>
+      <x:c r="F31" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="15.75">
+      <x:c r="A32" s="2" t="str">
         <x:v>Non-Unitary Quantum Machine Learning
 </x:v>
       </x:c>
-      <x:c r="B28" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C28" s="2" t="str">
+      <x:c r="B32" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D28" s="2" t="str">
+      <x:c r="D32" s="2" t="str">
         <x:v>Heredge, Jamie, et al.</x:v>
       </x:c>
-      <x:c r="E28" s="2" t="str">
+      <x:c r="E32" s="2" t="str">
         <x:v>https://arxiv.org/abs/2405.17388</x:v>
       </x:c>
-      <x:c r="F28" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="15.75">
-      <x:c r="A29" s="2" t="str">
+      <x:c r="F32" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="15.75">
+      <x:c r="A33" s="2" t="str">
         <x:v>Blockchain and Quantum Machine Learning Driven Energy Trading for Electric Vehicles
 </x:v>
       </x:c>
-      <x:c r="B29" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C29" s="2" t="str">
+      <x:c r="B33" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
         <x:v>Ad Hoc Networks </x:v>
       </x:c>
-      <x:c r="D29" s="2" t="str">
+      <x:c r="D33" s="2" t="str">
         <x:v>Kashyap, Pankaj Kumar, et al.</x:v>
       </x:c>
-      <x:c r="E29" s="2" t="str">
+      <x:c r="E33" s="2" t="str">
         <x:v>https://www.sciencedirect.com/science/article/abs/pii/S1570870524002439</x:v>
       </x:c>
-      <x:c r="F29" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="15.75">
-      <x:c r="A30" s="2" t="str">
+      <x:c r="F33" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="15.75">
+      <x:c r="A34" s="2" t="str">
         <x:v>
 Predicting Demand in Supply Chain Networks With Quantum Machine Learning Approach</x:v>
       </x:c>
-      <x:c r="B30" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C30" s="2" t="str">
+      <x:c r="B34" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C34" s="2" t="str">
         <x:v>. IGI Global</x:v>
       </x:c>
-      <x:c r="D30" s="2" t="str">
+      <x:c r="D34" s="2" t="str">
         <x:v>Sehrawat, Sunil Kumar, et al.</x:v>
       </x:c>
-      <x:c r="E30" s="2" t="str">
+      <x:c r="E34" s="2" t="str">
         <x:v>https://www.igi-global.com/chapter/predicting-demand-in-supply-chain-networks-with-quantum-machine-learning-approach/351811</x:v>
       </x:c>
-      <x:c r="F30" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="15.75">
-      <x:c r="A31" s="2" t="str">
+      <x:c r="F34" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="15.75">
+      <x:c r="A35" s="2" t="str">
         <x:v>
 AI-Infused Quantum Machine Learning for Enhanced Supply Chain Forecasting</x:v>
       </x:c>
-      <x:c r="B31" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C31" s="2" t="str">
+      <x:c r="B35" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="str">
         <x:v>. IGI Global</x:v>
       </x:c>
-      <x:c r="D31" s="2" t="str">
+      <x:c r="D35" s="2" t="str">
         <x:v>Gutta, Leela Manush, et al.</x:v>
       </x:c>
-      <x:c r="E31" s="2" t="str">
+      <x:c r="E35" s="2" t="str">
         <x:v>https://www.igi-global.com/chapter/ai-infused-quantum-machine-learning-for-enhanced-supply-chain-forecasting/351812</x:v>
       </x:c>
-      <x:c r="F31" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="15.75">
-      <x:c r="A32" s="2" t="str">
+      <x:c r="F35" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="15.75">
+      <x:c r="A36" s="2" t="str">
         <x:v>Dequantizing quantum machine learning models using tensor networks</x:v>
       </x:c>
-      <x:c r="B32" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C32" s="2" t="str">
+      <x:c r="B36" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C36" s="2" t="str">
         <x:v>Physical Review Research </x:v>
       </x:c>
-      <x:c r="D32" s="2" t="str">
+      <x:c r="D36" s="2" t="str">
         <x:v>Shin, Seongwook, Yong Siah Teo, and Hyunseok Jeong.</x:v>
       </x:c>
-      <x:c r="E32" s="2" t="str">
+      <x:c r="E36" s="2" t="str">
         <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.6.023218</x:v>
       </x:c>
-      <x:c r="F32" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="15.75">
-      <x:c r="A33" s="2" t="str">
+      <x:c r="F36" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="15.75">
+      <x:c r="A37" s="2" t="str">
         <x:v>Scalable quantum dynamics compilation via quantum machine learning</x:v>
       </x:c>
-      <x:c r="B33" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C33" s="2" t="str">
+      <x:c r="B37" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C37" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D33" s="2" t="str">
+      <x:c r="D37" s="2" t="str">
         <x:v>Zhang, Yuxuan, et al.</x:v>
       </x:c>
-      <x:c r="E33" s="2" t="str">
+      <x:c r="E37" s="2" t="str">
         <x:v>https://arxiv.org/abs/2409.16346</x:v>
       </x:c>
-      <x:c r="F33" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="15.75">
-      <x:c r="A34" s="2" t="str">
+      <x:c r="F37" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="15.75">
+      <x:c r="A38" s="2" t="str">
         <x:v>Financial fraud detection: a comparative study of quantum machine learning models</x:v>
       </x:c>
-      <x:c r="B34" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C34" s="2" t="str">
+      <x:c r="B38" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C38" s="2" t="str">
         <x:v>International Journal of Quantum Information </x:v>
       </x:c>
-      <x:c r="D34" s="2" t="str">
+      <x:c r="D38" s="2" t="str">
         <x:v>Innan, Nouhaila, Muhammad Al-Zafar Khan, and Mohamed Bennai.</x:v>
       </x:c>
-      <x:c r="E34" s="2" t="str">
+      <x:c r="E38" s="2" t="str">
         <x:v>https://www.worldscientific.com/doi/abs/10.1142/S0219749923500442?download=true&amp;journalCode=ijqi</x:v>
       </x:c>
-      <x:c r="F34" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="15.75">
-      <x:c r="A35" s="2" t="str">
+      <x:c r="F38" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="15.75">
+      <x:c r="A39" s="2" t="str">
         <x:v>Federated Quantum Machine Learning with Differential Privacy
 </x:v>
       </x:c>
-      <x:c r="B35" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C35" s="2" t="str">
+      <x:c r="B39" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C39" s="2" t="str">
         <x:v>IEEE International Conference on Acoustics, Speech and Signal Processing (ICASSP)</x:v>
       </x:c>
-      <x:c r="D35" s="2" t="str">
+      <x:c r="D39" s="2" t="str">
         <x:v>Rofougaran, Rod, et al.</x:v>
       </x:c>
-      <x:c r="E35" s="2" t="str">
+      <x:c r="E39" s="2" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10447155</x:v>
       </x:c>
-      <x:c r="F35" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="15.75">
-      <x:c r="A36" s="2" t="str">
+      <x:c r="F39" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="15.75">
+      <x:c r="A40" s="2" t="str">
         <x:v>Measurement-based quantum machine learning</x:v>
       </x:c>
-      <x:c r="B36" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C36" s="2" t="str">
+      <x:c r="B40" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C40" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D36" s="2" t="str">
+      <x:c r="D40" s="2" t="str">
         <x:v>Calderón, Luis Mantilla, et al.</x:v>
       </x:c>
-      <x:c r="E36" s="2" t="str">
+      <x:c r="E40" s="2" t="str">
         <x:v>https://arxiv.org/abs/2405.08319</x:v>
       </x:c>
-      <x:c r="F36" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="15.75">
-      <x:c r="A37" s="2" t="str">
+      <x:c r="F40" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="15.75">
+      <x:c r="A41" s="2" t="str">
         <x:v>Improving gradient methods via coordinate transformations: Applications to quantum machine learning
 </x:v>
       </x:c>
-      <x:c r="B37" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C37" s="2" t="str">
+      <x:c r="B41" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C41" s="2" t="str">
         <x:v>Physical Review Research </x:v>
       </x:c>
-      <x:c r="D37" s="2" t="str">
+      <x:c r="D41" s="2" t="str">
         <x:v>Bermejo, Pablo, Borja Aizpurua, and Román Orús.</x:v>
       </x:c>
-      <x:c r="E37" s="2" t="str">
+      <x:c r="E41" s="2" t="str">
         <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.6.023069</x:v>
       </x:c>
-      <x:c r="F37" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="15.75">
-      <x:c r="A38" s="2" t="str">
+      <x:c r="F41" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="15.75">
+      <x:c r="A42" s="2" t="str">
         <x:v>Predominant Aspects on Security for Quantum Machine Learning: Literature Review
 </x:v>
       </x:c>
-      <x:c r="B38" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C38" s="2" t="str">
+      <x:c r="B42" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C42" s="2" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D38" s="2" t="str">
+      <x:c r="D42" s="2" t="str">
         <x:v>Franco, Nicola, et al.</x:v>
       </x:c>
-      <x:c r="E38" s="2" t="str">
+      <x:c r="E42" s="2" t="str">
         <x:v>https://arxiv.org/abs/2401.07774</x:v>
       </x:c>
-      <x:c r="F38" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="15.75">
-      <x:c r="A39" s="2" t="str">
+      <x:c r="F42" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="15.75">
+      <x:c r="A43" s="2" t="str">
         <x:v>Innan, Nouhaila, et al. "Quantum state tomography using quantum machine learning." Quantum Machine Intelligence 6.1 (2024): 28.</x:v>
       </x:c>
-      <x:c r="B39" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C39" s="2" t="str">
+      <x:c r="B43" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C43" s="2" t="str">
         <x:v>Quantum Machine Intelligence</x:v>
       </x:c>
-      <x:c r="D39" s="2" t="str">
+      <x:c r="D43" s="2" t="str">
         <x:v>Innan, Nouhaila, et al.</x:v>
       </x:c>
-      <x:c r="E39" s="2" t="str">
+      <x:c r="E43" s="2" t="str">
         <x:v>https://link.springer.com/article/10.1007/s42484-024-00162-3</x:v>
       </x:c>
-      <x:c r="F39" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="15.75">
-      <x:c r="A40" s="2" t="str">
+      <x:c r="F43" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="15.75">
+      <x:c r="A44" s="2" t="str">
         <x:v>Improved financial forecasting via quantum machine learning</x:v>
       </x:c>
-      <x:c r="B40" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C40" s="2" t="str">
+      <x:c r="B44" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C44" s="2" t="str">
         <x:v>Quantum Machine Intelligence</x:v>
       </x:c>
-      <x:c r="D40" s="2" t="str">
+      <x:c r="D44" s="2" t="str">
         <x:v>Thakkar, Sohum, et al.</x:v>
       </x:c>
-      <x:c r="E40" s="2" t="str">
+      <x:c r="E44" s="2" t="str">
         <x:v>https://link.springer.com/article/10.1007/s42484-024-00157-0</x:v>
       </x:c>
-      <x:c r="F40" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="15.75">
-      <x:c r="A41" s="2" t="str">
+      <x:c r="F44" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="15.75">
+      <x:c r="A45" s="2" t="str">
         <x:v>Quantum Machine Learning for Credit Scoring
 </x:v>
       </x:c>
-      <x:c r="B41" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C41" s="2" t="str">
+      <x:c r="B45" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C45" s="2" t="str">
         <x:v>Mathematics</x:v>
       </x:c>
-      <x:c r="D41" s="2" t="str">
+      <x:c r="D45" s="2" t="str">
         <x:v>Schetakis, Nikolaos, et al.</x:v>
       </x:c>
-      <x:c r="E41" s="2" t="str">
+      <x:c r="E45" s="2" t="str">
         <x:v>https://www.mdpi.com/2227-7390/12/9/1391</x:v>
       </x:c>
-      <x:c r="F41" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="15.75">
-      <x:c r="A42" s="2" t="str">
+      <x:c r="F45" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="15.75">
+      <x:c r="A46" s="2" t="str">
         <x:v>A comparative and practical approach using quantum machine learning (QML) and support vector classifier (SVC) for Light emitting diodes mediated in vitro micropropagation of black mulberry (Morus nigra L.)</x:v>
       </x:c>
-      <x:c r="B42" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C42" s="2" t="str">
+      <x:c r="B46" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C46" s="2" t="str">
         <x:v>Industrial Crops and Products </x:v>
       </x:c>
-      <x:c r="D42" s="2" t="str">
+      <x:c r="D46" s="2" t="str">
         <x:v>Aasim, Muhammad, et al.</x:v>
       </x:c>
-      <x:c r="E42" s="2" t="str">
+      <x:c r="E46" s="2" t="str">
         <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0926669024003741</x:v>
       </x:c>
-      <x:c r="F42" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="15.75">
-      <x:c r="A43" s="2" t="str">
+      <x:c r="F46" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="15.75">
+      <x:c r="A47" s="2" t="str">
         <x:v>Variational quantum circuit-based quantum machine learning approach for predicting corrosion inhibition efficiency of pyridine-quinoline compounds</x:v>
       </x:c>
-      <x:c r="B43" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C43" s="2" t="str">
+      <x:c r="B47" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C47" s="2" t="str">
         <x:v>Materials Today Quantum </x:v>
       </x:c>
-      <x:c r="D43" s="2" t="str">
+      <x:c r="D47" s="2" t="str">
         <x:v>Akrom, Muhamad, Supriadi Rustad, and Hermawan Kresno Dipojono.</x:v>
       </x:c>
-      <x:c r="E43" s="2" t="str">
+      <x:c r="E47" s="2" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S2950257824000076</x:v>
       </x:c>
-      <x:c r="F43" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="15.75">
-      <x:c r="A44" s="2" t="str">
+      <x:c r="F47" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="15.75">
+      <x:c r="A48" s="2" t="str">
         <x:v>A parallel quantum eigensolver for quantum machine learning
 </x:v>
       </x:c>
-      <x:c r="B44" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C44" s="2" t="str">
+      <x:c r="B48" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C48" s="2" t="str">
         <x:v>New Journal of Physics </x:v>
       </x:c>
-      <x:c r="D44" s="2" t="str">
+      <x:c r="D48" s="2" t="str">
         <x:v>Yang, Fan, et al.</x:v>
       </x:c>
-      <x:c r="E44" s="2" t="str">
+      <x:c r="E48" s="2" t="str">
         <x:v>https://iopscience.iop.org/article/10.1088/1367-2630/ad15b4/meta</x:v>
-      </x:c>
-      <x:c r="F44" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="15.75">
-      <x:c r="A45" s="2" t="str">
-        <x:v>Quantum machine learning-based framework to detect heart failures in Healthcare 4.0</x:v>
-      </x:c>
-      <x:c r="B45" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C45" s="2" t="str">
-        <x:v>Software: Practice and Experience </x:v>
-      </x:c>
-      <x:c r="D45" s="2" t="str">
-        <x:v>Munshi, Manushi, et al.</x:v>
-      </x:c>
-      <x:c r="E45" s="2" t="str">
-        <x:v>https://onlinelibrary.wiley.com/doi/abs/10.1002/spe.3264</x:v>
-      </x:c>
-      <x:c r="F45" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46" ht="15.75">
-      <x:c r="A46" s="2" t="str">
-        <x:v>A comprehensive approach utilizing quantum machine learning in the study of corrosion inhibition on quinoxaline compounds</x:v>
-      </x:c>
-      <x:c r="B46" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C46" s="2" t="str">
-        <x:v>Artificial Intelligence Chemistry </x:v>
-      </x:c>
-      <x:c r="D46" s="2" t="str">
-        <x:v>Akrom, Muhamad, et al.</x:v>
-      </x:c>
-      <x:c r="E46" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/pii/S2949747724000319</x:v>
-      </x:c>
-      <x:c r="F46" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47" ht="15.75">
-      <x:c r="A47" s="2" t="str">
-        <x:v>Quantum Machine Learning Playground</x:v>
-      </x:c>
-      <x:c r="B47" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C47" s="2" t="str">
-        <x:v>IEEE Computer Graphics and Applications</x:v>
-      </x:c>
-      <x:c r="D47" s="2" t="str">
-        <x:v>Debus, Pascal, Sebastian Issel, and Kilian Tscharke.</x:v>
-      </x:c>
-      <x:c r="E47" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10669759</x:v>
-      </x:c>
-      <x:c r="F47" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48" ht="15.75">
-      <x:c r="A48" s="2" t="str">
-        <x:v>Transition role of entangled data in quantum machine learning</x:v>
-      </x:c>
-      <x:c r="B48" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C48" s="2" t="str">
-        <x:v>Nature Communications </x:v>
-      </x:c>
-      <x:c r="D48" s="2" t="str">
-        <x:v>Wang, Xinbiao, et al.</x:v>
-      </x:c>
-      <x:c r="E48" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s41467-024-47983-1</x:v>
       </x:c>
       <x:c r="F48" s="2" t="str">
         <x:v>QML</x:v>
@@ -1502,19 +1502,19 @@
     </x:row>
     <x:row r="49" ht="15.75">
       <x:c r="A49" s="2" t="str">
-        <x:v>Permutation invariant encodings for quantum machine learning with point cloud data</x:v>
+        <x:v>Quantum machine learning-based framework to detect heart failures in Healthcare 4.0</x:v>
       </x:c>
       <x:c r="B49" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C49" s="2" t="str">
-        <x:v>Quantum Machine Intelligence</x:v>
+        <x:v>Software: Practice and Experience </x:v>
       </x:c>
       <x:c r="D49" s="2" t="str">
-        <x:v>Heredge, Jamie, et al.</x:v>
+        <x:v>Munshi, Manushi, et al.</x:v>
       </x:c>
       <x:c r="E49" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s42484-024-00156-1</x:v>
+        <x:v>https://onlinelibrary.wiley.com/doi/abs/10.1002/spe.3264</x:v>
       </x:c>
       <x:c r="F49" s="2" t="str">
         <x:v>QML</x:v>
@@ -1522,98 +1522,100 @@
     </x:row>
     <x:row r="50" ht="15.75">
       <x:c r="A50" s="2" t="str">
+        <x:v>A comprehensive approach utilizing quantum machine learning in the study of corrosion inhibition on quinoxaline compounds</x:v>
+      </x:c>
+      <x:c r="B50" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C50" s="2" t="str">
+        <x:v>Artificial Intelligence Chemistry </x:v>
+      </x:c>
+      <x:c r="D50" s="2" t="str">
+        <x:v>Akrom, Muhamad, et al.</x:v>
+      </x:c>
+      <x:c r="E50" s="2" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/pii/S2949747724000319</x:v>
+      </x:c>
+      <x:c r="F50" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="15.75">
+      <x:c r="A51" s="2" t="str">
+        <x:v>Quantum Machine Learning Playground</x:v>
+      </x:c>
+      <x:c r="B51" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C51" s="2" t="str">
+        <x:v>IEEE Computer Graphics and Applications</x:v>
+      </x:c>
+      <x:c r="D51" s="2" t="str">
+        <x:v>Debus, Pascal, Sebastian Issel, and Kilian Tscharke.</x:v>
+      </x:c>
+      <x:c r="E51" s="2" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10669759</x:v>
+      </x:c>
+      <x:c r="F51" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="15.75">
+      <x:c r="A52" s="2" t="str">
+        <x:v>Transition role of entangled data in quantum machine learning</x:v>
+      </x:c>
+      <x:c r="B52" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C52" s="2" t="str">
+        <x:v>Nature Communications </x:v>
+      </x:c>
+      <x:c r="D52" s="2" t="str">
+        <x:v>Wang, Xinbiao, et al.</x:v>
+      </x:c>
+      <x:c r="E52" s="2" t="str">
+        <x:v>https://www.nature.com/articles/s41467-024-47983-1</x:v>
+      </x:c>
+      <x:c r="F52" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="15.75">
+      <x:c r="A53" s="2" t="str">
+        <x:v>Permutation invariant encodings for quantum machine learning with point cloud data</x:v>
+      </x:c>
+      <x:c r="B53" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C53" s="2" t="str">
+        <x:v>Quantum Machine Intelligence</x:v>
+      </x:c>
+      <x:c r="D53" s="2" t="str">
+        <x:v>Heredge, Jamie, et al.</x:v>
+      </x:c>
+      <x:c r="E53" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s42484-024-00156-1</x:v>
+      </x:c>
+      <x:c r="F53" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="15.75">
+      <x:c r="A54" s="2" t="str">
         <x:v>Encoding optimization for quantum machine learning demonstrated on a superconducting transmon qutrit
 </x:v>
       </x:c>
-      <x:c r="B50" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C50" s="2" t="str">
+      <x:c r="B54" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C54" s="2" t="str">
         <x:v>Quantum Science and Technology </x:v>
       </x:c>
-      <x:c r="D50" s="2" t="str">
+      <x:c r="D54" s="2" t="str">
         <x:v>Cao, Shuxiang, et al.</x:v>
       </x:c>
-      <x:c r="E50" s="2" t="str">
+      <x:c r="E54" s="2" t="str">
         <x:v>https://iopscience.iop.org/article/10.1088/2058-9565/ad7315/meta</x:v>
-      </x:c>
-      <x:c r="F50" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51" ht="15.75">
-      <x:c r="A51" s="2" t="str">
-        <x:v>A new quantum machine learning algorithm: split hidden quantum Markov model inspired by quantum conditional master equation.</x:v>
-      </x:c>
-      <x:c r="B51" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C51" s="2" t="str">
-        <x:v>Quantum</x:v>
-      </x:c>
-      <x:c r="D51" s="2" t="str">
-        <x:v>Li, Xiao-Yu, et al.</x:v>
-      </x:c>
-      <x:c r="E51" s="2"/>
-      <x:c r="F51" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52" ht="15.75">
-      <x:c r="A52" s="2" t="str">
-        <x:v>Alleviating Barren Plateaus in Parameterized Quantum Machine Learning Circuits: Investigating Advanced Parameter Initialization Strategies</x:v>
-      </x:c>
-      <x:c r="B52" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C52" s="2" t="str">
-        <x:v>Design, Automation &amp; Test in Europe Conference &amp; Exhibition (DATE)</x:v>
-      </x:c>
-      <x:c r="D52" s="2" t="str">
-        <x:v>Kashif, Muhammad, et al.</x:v>
-      </x:c>
-      <x:c r="E52" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10546644</x:v>
-      </x:c>
-      <x:c r="F52" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53" ht="15.75">
-      <x:c r="A53" s="2" t="str">
-        <x:v>Variational quantum approximate support vector machine with inference transfer</x:v>
-      </x:c>
-      <x:c r="B53" s="2" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C53" s="2" t="str">
-        <x:v>Scientific reports</x:v>
-      </x:c>
-      <x:c r="D53" s="2" t="str">
-        <x:v>Siheon Park, Daniel K. Park, June-Koo Kevin Rhee</x:v>
-      </x:c>
-      <x:c r="E53" s="2" t="str">
-        <x:v>https://doi.org/10.1038/s41598-023-29495-y</x:v>
-      </x:c>
-      <x:c r="F53" s="2" t="str">
-        <x:v>QML</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54" ht="15.75">
-      <x:c r="A54" s="2" t="str">
-        <x:v>Quantum Machine Learning: A Review and Case Studies</x:v>
-      </x:c>
-      <x:c r="B54" s="2" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C54" s="2" t="str">
-        <x:v>MDPI</x:v>
-      </x:c>
-      <x:c r="D54" s="2" t="str">
-        <x:v>Amine Zeguendry, Zahi Jarir, Mohamed Quafafou</x:v>
-      </x:c>
-      <x:c r="E54" s="2" t="str">
-        <x:v>https://doi.org/10.3390/e25020287</x:v>
       </x:c>
       <x:c r="F54" s="2" t="str">
         <x:v>QML</x:v>
@@ -1621,39 +1623,37 @@
     </x:row>
     <x:row r="55" ht="15.75">
       <x:c r="A55" s="2" t="str">
-        <x:v>Benchmarking adversarially robust quantum machine learning at scale</x:v>
+        <x:v>A new quantum machine learning algorithm: split hidden quantum Markov model inspired by quantum conditional master equation.</x:v>
       </x:c>
       <x:c r="B55" s="2" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C55" s="2" t="str">
-        <x:v>APS : Physical Review Research</x:v>
+        <x:v>Quantum</x:v>
       </x:c>
       <x:c r="D55" s="2" t="str">
-        <x:v>Maxwell T. West, Sarah M. Erfani, Christopher Leckie, Martin Sevior, Lloyd C. L. Hollenberg, Muhammad Usman</x:v>
-      </x:c>
-      <x:c r="E55" s="2" t="str">
-        <x:v>https://doi.org/10.1103/PhysRevResearch.5.023186</x:v>
-      </x:c>
+        <x:v>Li, Xiao-Yu, et al.</x:v>
+      </x:c>
+      <x:c r="E55" s="2"/>
       <x:c r="F55" s="2" t="str">
         <x:v>QML</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15.75">
       <x:c r="A56" s="2" t="str">
-        <x:v>Learning lattice quantum field theories with equivariant continuous flows</x:v>
+        <x:v>Alleviating Barren Plateaus in Parameterized Quantum Machine Learning Circuits: Investigating Advanced Parameter Initialization Strategies</x:v>
       </x:c>
       <x:c r="B56" s="2" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C56" s="2" t="str">
-        <x:v>SciPost</x:v>
+        <x:v>Design, Automation &amp; Test in Europe Conference &amp; Exhibition (DATE)</x:v>
       </x:c>
       <x:c r="D56" s="2" t="str">
-        <x:v>Mathis Gerdes, Pim de Haan, Corrado Rainone, Roberto Bondesan, Miranda C. N. Cheng</x:v>
+        <x:v>Kashif, Muhammad, et al.</x:v>
       </x:c>
       <x:c r="E56" s="2" t="str">
-        <x:v>https://doi.org/10.21468/SciPostPhys.15.6.238</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10546644</x:v>
       </x:c>
       <x:c r="F56" s="2" t="str">
         <x:v>QML</x:v>
@@ -1661,19 +1661,19 @@
     </x:row>
     <x:row r="57" ht="15.75">
       <x:c r="A57" s="2" t="str">
-        <x:v>Quantum machine learning in medical image analysis: A survey</x:v>
+        <x:v>Variational quantum approximate support vector machine with inference transfer</x:v>
       </x:c>
       <x:c r="B57" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C57" s="2" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>Scientific reports</x:v>
       </x:c>
       <x:c r="D57" s="2" t="str">
-        <x:v>Lin Wei, Haowen Liu, Jing Xu, Lei Shi, Zheng Shan, Bo Zhao, Yufei Gao</x:v>
+        <x:v>Siheon Park, Daniel K. Park, June-Koo Kevin Rhee</x:v>
       </x:c>
       <x:c r="E57" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.neucom.2023.01.049</x:v>
+        <x:v>https://doi.org/10.1038/s41598-023-29495-y</x:v>
       </x:c>
       <x:c r="F57" s="2" t="str">
         <x:v>QML</x:v>
@@ -1681,19 +1681,19 @@
     </x:row>
     <x:row r="58" ht="15.75">
       <x:c r="A58" s="2" t="str">
-        <x:v>Quantum angle encoding with learnable rotation applied to quantum–classical convolutional neural networks</x:v>
+        <x:v>Quantum Machine Learning: A Review and Case Studies</x:v>
       </x:c>
       <x:c r="B58" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C58" s="2" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D58" s="2" t="str">
-        <x:v>Emmanuel Ovalle-Magallanes, Dora E. Alvarado-Carrillo, Juan Gabriel Avina-Cervantes, van Cruz-Aceves, Jose Ruiz-Pinales</x:v>
+        <x:v>Amine Zeguendry, Zahi Jarir, Mohamed Quafafou</x:v>
       </x:c>
       <x:c r="E58" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.asoc.2023.110307</x:v>
+        <x:v>https://doi.org/10.3390/e25020287</x:v>
       </x:c>
       <x:c r="F58" s="2" t="str">
         <x:v>QML</x:v>
@@ -1701,19 +1701,19 @@
     </x:row>
     <x:row r="59" ht="15.75">
       <x:c r="A59" s="2" t="str">
-        <x:v>Similarity-based parameter transferability in the quantum approximate optimization algorithm</x:v>
+        <x:v>Benchmarking adversarially robust quantum machine learning at scale</x:v>
       </x:c>
       <x:c r="B59" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C59" s="2" t="str">
-        <x:v>frontiers</x:v>
+        <x:v>APS : Physical Review Research</x:v>
       </x:c>
       <x:c r="D59" s="2" t="str">
-        <x:v>Alexey Galda, Eesh Gupta, Jose Falla, Xiaoyuan Liu, Danylo Lykov, Yuri Alexeev, Ilya Safro</x:v>
+        <x:v>Maxwell T. West, Sarah M. Erfani, Christopher Leckie, Martin Sevior, Lloyd C. L. Hollenberg, Muhammad Usman</x:v>
       </x:c>
       <x:c r="E59" s="2" t="str">
-        <x:v>https://doi.org/10.3389/frqst.2023.1200975</x:v>
+        <x:v>https://doi.org/10.1103/PhysRevResearch.5.023186</x:v>
       </x:c>
       <x:c r="F59" s="2" t="str">
         <x:v>QML</x:v>
@@ -1721,19 +1721,19 @@
     </x:row>
     <x:row r="60" ht="15.75">
       <x:c r="A60" s="2" t="str">
-        <x:v>Learning quantum systems</x:v>
+        <x:v>Learning lattice quantum field theories with equivariant continuous flows</x:v>
       </x:c>
       <x:c r="B60" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C60" s="2" t="str">
-        <x:v>nature review</x:v>
+        <x:v>SciPost</x:v>
       </x:c>
       <x:c r="D60" s="2" t="str">
-        <x:v>Valentin Gebhart, Raffaele Santagati, Antonio Andrea Gentile, Erik M. Gauger, David Craig, Natalia Ares, Leonardo Banchi, Florian Marquardt, Luca Pezzè, Cristian Bonato</x:v>
+        <x:v>Mathis Gerdes, Pim de Haan, Corrado Rainone, Roberto Bondesan, Miranda C. N. Cheng</x:v>
       </x:c>
       <x:c r="E60" s="2" t="str">
-        <x:v>https://doi.org/10.1038/s42254-022-00552-1</x:v>
+        <x:v>https://doi.org/10.21468/SciPostPhys.15.6.238</x:v>
       </x:c>
       <x:c r="F60" s="2" t="str">
         <x:v>QML</x:v>
@@ -1741,7 +1741,7 @@
     </x:row>
     <x:row r="61" ht="15.75">
       <x:c r="A61" s="2" t="str">
-        <x:v>Advances in Quantum Machine Learning and Deep Learning for Image Classification: A Survey</x:v>
+        <x:v>Quantum machine learning in medical image analysis: A survey</x:v>
       </x:c>
       <x:c r="B61" s="2" t="n">
         <x:v>2023</x:v>
@@ -1750,10 +1750,10 @@
         <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D61" s="2" t="str">
-        <x:v>Ruba Kharsa,  Ahmed Bouridane,  Abbes Amira</x:v>
+        <x:v>Lin Wei, Haowen Liu, Jing Xu, Lei Shi, Zheng Shan, Bo Zhao, Yufei Gao</x:v>
       </x:c>
       <x:c r="E61" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.neucom.2023.126843</x:v>
+        <x:v>https://doi.org/10.1016/j.neucom.2023.01.049</x:v>
       </x:c>
       <x:c r="F61" s="2" t="str">
         <x:v>QML</x:v>
@@ -1761,19 +1761,19 @@
     </x:row>
     <x:row r="62" ht="15.75">
       <x:c r="A62" s="2" t="str">
-        <x:v>Hybrid quantum ResNet for car classification and its hyperparameter optimization</x:v>
+        <x:v>Quantum angle encoding with learnable rotation applied to quantum–classical convolutional neural networks</x:v>
       </x:c>
       <x:c r="B62" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C62" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D62" s="2" t="str">
-        <x:v>Asel Sagingalieva, Mo Kordzanganeh, Andrii Kurkin, Artem Melnikov, Daniil Kuhmistrov, Michael Perelshtein, Alexey Melnikov, Andrea Skolik, David Von Dollen</x:v>
+        <x:v>Emmanuel Ovalle-Magallanes, Dora E. Alvarado-Carrillo, Juan Gabriel Avina-Cervantes, van Cruz-Aceves, Jose Ruiz-Pinales</x:v>
       </x:c>
       <x:c r="E62" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00123-2</x:v>
+        <x:v>https://doi.org/10.1016/j.asoc.2023.110307</x:v>
       </x:c>
       <x:c r="F62" s="2" t="str">
         <x:v>QML</x:v>
@@ -1781,19 +1781,19 @@
     </x:row>
     <x:row r="63" ht="15.75">
       <x:c r="A63" s="2" t="str">
-        <x:v>Parameter Transfer for Quantum Approximate Optimization of Weighted MaxCut</x:v>
+        <x:v>Similarity-based parameter transferability in the quantum approximate optimization algorithm</x:v>
       </x:c>
       <x:c r="B63" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C63" s="2" t="str">
-        <x:v>ACM</x:v>
+        <x:v>frontiers</x:v>
       </x:c>
       <x:c r="D63" s="2" t="str">
-        <x:v>Ruslan Shaydulin, Phillip C. Lotshaw, Jeffrey Larson, James Ostrowski, Travis S. Humble</x:v>
+        <x:v>Alexey Galda, Eesh Gupta, Jose Falla, Xiaoyuan Liu, Danylo Lykov, Yuri Alexeev, Ilya Safro</x:v>
       </x:c>
       <x:c r="E63" s="2" t="str">
-        <x:v>https://doi.org/10.1145/3584706</x:v>
+        <x:v>https://doi.org/10.3389/frqst.2023.1200975</x:v>
       </x:c>
       <x:c r="F63" s="2" t="str">
         <x:v>QML</x:v>
@@ -1801,19 +1801,19 @@
     </x:row>
     <x:row r="64" ht="15.75">
       <x:c r="A64" s="2" t="str">
-        <x:v>Foundations of Quantum Federated Learning Over Classical and Quantum Networks</x:v>
+        <x:v>Learning quantum systems</x:v>
       </x:c>
       <x:c r="B64" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C64" s="2" t="str">
-        <x:v>IEEE</x:v>
+        <x:v>nature review</x:v>
       </x:c>
       <x:c r="D64" s="2" t="str">
-        <x:v>Mahdi Chehimi, Samuel Yen-Chi Chen, Walid Saad, Don Towsley, Mérouane Debbah</x:v>
+        <x:v>Valentin Gebhart, Raffaele Santagati, Antonio Andrea Gentile, Erik M. Gauger, David Craig, Natalia Ares, Leonardo Banchi, Florian Marquardt, Luca Pezzè, Cristian Bonato</x:v>
       </x:c>
       <x:c r="E64" s="2" t="str">
-        <x:v>https://doi.org/10.1109/MNET.2023.3327365</x:v>
+        <x:v>https://doi.org/10.1038/s42254-022-00552-1</x:v>
       </x:c>
       <x:c r="F64" s="2" t="str">
         <x:v>QML</x:v>
@@ -1821,19 +1821,19 @@
     </x:row>
     <x:row r="65" ht="15.75">
       <x:c r="A65" s="2" t="str">
-        <x:v>Quantum machine learning with differential privacy</x:v>
+        <x:v>Advances in Quantum Machine Learning and Deep Learning for Image Classification: A Survey</x:v>
       </x:c>
       <x:c r="B65" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C65" s="2" t="str">
-        <x:v>Scientific reports</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D65" s="2" t="str">
-        <x:v>William M. Watkins, Samuel Yen-Chi Chen, Shinjae Yoo</x:v>
+        <x:v>Ruba Kharsa,  Ahmed Bouridane,  Abbes Amira</x:v>
       </x:c>
       <x:c r="E65" s="2" t="str">
-        <x:v>https://doi.org/10.1038/s41598-022-24082-z</x:v>
+        <x:v>https://doi.org/10.1016/j.neucom.2023.126843</x:v>
       </x:c>
       <x:c r="F65" s="2" t="str">
         <x:v>QML</x:v>
@@ -1841,19 +1841,19 @@
     </x:row>
     <x:row r="66" ht="15.75">
       <x:c r="A66" s="2" t="str">
-        <x:v>Out-of-distribution generalization for learning quantum dynamics</x:v>
+        <x:v>Hybrid quantum ResNet for car classification and its hyperparameter optimization</x:v>
       </x:c>
       <x:c r="B66" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C66" s="2" t="str">
-        <x:v>nature communication</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D66" s="2" t="str">
-        <x:v>Matthias C. Caro, Hsin-Yuan Huang, Nicholas Ezzell, Joe Gibbs, Andrew T. Sornborger, Lukasz Cincio, Patrick J. Coles, Zoë Holmes </x:v>
+        <x:v>Asel Sagingalieva, Mo Kordzanganeh, Andrii Kurkin, Artem Melnikov, Daniil Kuhmistrov, Michael Perelshtein, Alexey Melnikov, Andrea Skolik, David Von Dollen</x:v>
       </x:c>
       <x:c r="E66" s="2" t="str">
-        <x:v>https://doi.org/10.1038/s41467-023-39381-w</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00123-2</x:v>
       </x:c>
       <x:c r="F66" s="2" t="str">
         <x:v>QML</x:v>
@@ -1861,19 +1861,19 @@
     </x:row>
     <x:row r="67" ht="15.75">
       <x:c r="A67" s="2" t="str">
-        <x:v>Exploiting Symmetry in Variational Quantum Machine Learning</x:v>
+        <x:v>Parameter Transfer for Quantum Approximate Optimization of Weighted MaxCut</x:v>
       </x:c>
       <x:c r="B67" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C67" s="2" t="str">
-        <x:v>APS : PRX QUANTUM</x:v>
+        <x:v>ACM</x:v>
       </x:c>
       <x:c r="D67" s="2" t="str">
-        <x:v>Johannes Jakob Meyer, Marian Mularski, Elies Gil-Fuster, Antonio Anna Mele, Francesco Arzani, Alissa Wilms,  Jens Eisert</x:v>
+        <x:v>Ruslan Shaydulin, Phillip C. Lotshaw, Jeffrey Larson, James Ostrowski, Travis S. Humble</x:v>
       </x:c>
       <x:c r="E67" s="2" t="str">
-        <x:v>https://doi.org/10.1103/PRXQuantum.4.010328</x:v>
+        <x:v>https://doi.org/10.1145/3584706</x:v>
       </x:c>
       <x:c r="F67" s="2" t="str">
         <x:v>QML</x:v>
@@ -1881,19 +1881,19 @@
     </x:row>
     <x:row r="68" ht="15.75">
       <x:c r="A68" s="2" t="str">
-        <x:v>Machine learning quantum mechanical ground states based on stochastic mechanics</x:v>
+        <x:v>Foundations of Quantum Federated Learning Over Classical and Quantum Networks</x:v>
       </x:c>
       <x:c r="B68" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C68" s="2" t="str">
-        <x:v>APS : Physical Review A covering atomic, molecular, and optical physics and quantum science</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D68" s="2" t="str">
-        <x:v>Kai-Hendrik Henk, Wolfgang Paul</x:v>
+        <x:v>Mahdi Chehimi, Samuel Yen-Chi Chen, Walid Saad, Don Towsley, Mérouane Debbah</x:v>
       </x:c>
       <x:c r="E68" s="2" t="str">
-        <x:v>https://doi.org/10.1103/PhysRevA.108.062412</x:v>
+        <x:v>https://doi.org/10.1109/MNET.2023.3327365</x:v>
       </x:c>
       <x:c r="F68" s="2" t="str">
         <x:v>QML</x:v>
@@ -1901,19 +1901,19 @@
     </x:row>
     <x:row r="69" ht="15.75">
       <x:c r="A69" s="2" t="str">
-        <x:v>Quantum-probabilistic Hamiltonian learning for generative modeling and anomaly detection</x:v>
+        <x:v>Quantum machine learning with differential privacy</x:v>
       </x:c>
       <x:c r="B69" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C69" s="2" t="str">
-        <x:v>APS : Physical Review A covering atomic, molecular, and optical physics and quantum science</x:v>
+        <x:v>Scientific reports</x:v>
       </x:c>
       <x:c r="D69" s="2" t="str">
-        <x:v>Jack Y. Araz and Michael Spannowsky</x:v>
+        <x:v>William M. Watkins, Samuel Yen-Chi Chen, Shinjae Yoo</x:v>
       </x:c>
       <x:c r="E69" s="2" t="str">
-        <x:v>https://doi.org/10.1103/PhysRevA.108.062422</x:v>
+        <x:v>https://doi.org/10.1038/s41598-022-24082-z</x:v>
       </x:c>
       <x:c r="F69" s="2" t="str">
         <x:v>QML</x:v>
@@ -1921,19 +1921,19 @@
     </x:row>
     <x:row r="70" ht="15.75">
       <x:c r="A70" s="2" t="str">
-        <x:v>A semi-agnostic ansatz with variable structure for variational quantum algorithms</x:v>
+        <x:v>Out-of-distribution generalization for learning quantum dynamics</x:v>
       </x:c>
       <x:c r="B70" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C70" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>nature communication</x:v>
       </x:c>
       <x:c r="D70" s="2" t="str">
-        <x:v>M. Bilkis, M. Cerezo, Guillaume Verdon, Patrick J. Coles, Lukasz Cincio</x:v>
+        <x:v>Matthias C. Caro, Hsin-Yuan Huang, Nicholas Ezzell, Joe Gibbs, Andrew T. Sornborger, Lukasz Cincio, Patrick J. Coles, Zoë Holmes </x:v>
       </x:c>
       <x:c r="E70" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00132-1</x:v>
+        <x:v>https://doi.org/10.1038/s41467-023-39381-w</x:v>
       </x:c>
       <x:c r="F70" s="2" t="str">
         <x:v>QML</x:v>
@@ -1941,19 +1941,19 @@
     </x:row>
     <x:row r="71" ht="15.75">
       <x:c r="A71" s="2" t="str">
-        <x:v>A hybrid quantum-classical approach for inference on restricted Boltzmann machines</x:v>
+        <x:v>Exploiting Symmetry in Variational Quantum Machine Learning</x:v>
       </x:c>
       <x:c r="B71" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C71" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>APS : PRX QUANTUM</x:v>
       </x:c>
       <x:c r="D71" s="2" t="str">
-        <x:v>Mārtiņš Kālis, Andris Locāns, Rolands Šikovs, Hassan Naseri, Andris Ambainis</x:v>
+        <x:v>Johannes Jakob Meyer, Marian Mularski, Elies Gil-Fuster, Antonio Anna Mele, Francesco Arzani, Alissa Wilms,  Jens Eisert</x:v>
       </x:c>
       <x:c r="E71" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00135-y</x:v>
+        <x:v>https://doi.org/10.1103/PRXQuantum.4.010328</x:v>
       </x:c>
       <x:c r="F71" s="2" t="str">
         <x:v>QML</x:v>
@@ -1961,19 +1961,19 @@
     </x:row>
     <x:row r="72" ht="15.75">
       <x:c r="A72" s="2" t="str">
-        <x:v>Time series quantum classifiers with amplitude embedding</x:v>
+        <x:v>Machine learning quantum mechanical ground states based on stochastic mechanics</x:v>
       </x:c>
       <x:c r="B72" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C72" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>APS : Physical Review A covering atomic, molecular, and optical physics and quantum science</x:v>
       </x:c>
       <x:c r="D72" s="2" t="str">
-        <x:v>M. P. Cuéllar, C. Cano, L. G. B. Ruiz, L. Servadei</x:v>
+        <x:v>Kai-Hendrik Henk, Wolfgang Paul</x:v>
       </x:c>
       <x:c r="E72" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00133-0</x:v>
+        <x:v>https://doi.org/10.1103/PhysRevA.108.062412</x:v>
       </x:c>
       <x:c r="F72" s="2" t="str">
         <x:v>QML</x:v>
@@ -1981,19 +1981,19 @@
     </x:row>
     <x:row r="73" ht="15.75">
       <x:c r="A73" s="2" t="str">
-        <x:v>The cross-sectional stock return predictions via quantum neural network and tensor network</x:v>
+        <x:v>Quantum-probabilistic Hamiltonian learning for generative modeling and anomaly detection</x:v>
       </x:c>
       <x:c r="B73" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C73" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>APS : Physical Review A covering atomic, molecular, and optical physics and quantum science</x:v>
       </x:c>
       <x:c r="D73" s="2" t="str">
-        <x:v>Nozomu Kobayashi, Yoshiyuki Suimon, Koichi Miyamoto, Kosuke Mitarai</x:v>
+        <x:v>Jack Y. Araz and Michael Spannowsky</x:v>
       </x:c>
       <x:c r="E73" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00136-x</x:v>
+        <x:v>https://doi.org/10.1103/PhysRevA.108.062422</x:v>
       </x:c>
       <x:c r="F73" s="2" t="str">
         <x:v>QML</x:v>
@@ -2001,7 +2001,7 @@
     </x:row>
     <x:row r="74" ht="15.75">
       <x:c r="A74" s="2" t="str">
-        <x:v>A quantum “black box” for entropy calculation</x:v>
+        <x:v>A semi-agnostic ansatz with variable structure for variational quantum algorithms</x:v>
       </x:c>
       <x:c r="B74" s="2" t="n">
         <x:v>2023</x:v>
@@ -2010,10 +2010,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D74" s="2" t="str">
-        <x:v>Michal Koren, Oded Koren, Or Peretz</x:v>
+        <x:v>M. Bilkis, M. Cerezo, Guillaume Verdon, Patrick J. Coles, Lukasz Cincio</x:v>
       </x:c>
       <x:c r="E74" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00127-y</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00132-1</x:v>
       </x:c>
       <x:c r="F74" s="2" t="str">
         <x:v>QML</x:v>
@@ -2021,7 +2021,7 @@
     </x:row>
     <x:row r="75" ht="15.75">
       <x:c r="A75" s="2" t="str">
-        <x:v>Data re-uploading with a single qudit</x:v>
+        <x:v>A hybrid quantum-classical approach for inference on restricted Boltzmann machines</x:v>
       </x:c>
       <x:c r="B75" s="2" t="n">
         <x:v>2023</x:v>
@@ -2030,10 +2030,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D75" s="2" t="str">
-        <x:v>Noah L. Wach, Manuel S. Rudolph, Fred Jendrzejewski, Sebastian Schmitt</x:v>
+        <x:v>Mārtiņš Kālis, Andris Locāns, Rolands Šikovs, Hassan Naseri, Andris Ambainis</x:v>
       </x:c>
       <x:c r="E75" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00125-0</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00135-y</x:v>
       </x:c>
       <x:c r="F75" s="2" t="str">
         <x:v>QML</x:v>
@@ -2041,7 +2041,7 @@
     </x:row>
     <x:row r="76" ht="15.75">
       <x:c r="A76" s="2" t="str">
-        <x:v>Comparing quantum and classical machine learning for Vector Boson Scattering background reduction at the Large Hadron Collider</x:v>
+        <x:v>Time series quantum classifiers with amplitude embedding</x:v>
       </x:c>
       <x:c r="B76" s="2" t="n">
         <x:v>2023</x:v>
@@ -2050,10 +2050,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D76" s="2" t="str">
-        <x:v>Davide Cugini, Dario Gerace, Pietro Govoni, Aurora Perego, Davide Valsecchi </x:v>
+        <x:v>M. P. Cuéllar, C. Cano, L. G. B. Ruiz, L. Servadei</x:v>
       </x:c>
       <x:c r="E76" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00106-3</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00133-0</x:v>
       </x:c>
       <x:c r="F76" s="2" t="str">
         <x:v>QML</x:v>
@@ -2061,7 +2061,7 @@
     </x:row>
     <x:row r="77" ht="15.75">
       <x:c r="A77" s="2" t="str">
-        <x:v>Classical splitting of parametrized quantum circuits</x:v>
+        <x:v>The cross-sectional stock return predictions via quantum neural network and tensor network</x:v>
       </x:c>
       <x:c r="B77" s="2" t="n">
         <x:v>2023</x:v>
@@ -2070,10 +2070,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D77" s="2" t="str">
-        <x:v>Cenk Tüysüz, Giuseppe Clemente, Arianna Crippa, Tobias Hartung, Stefan Kühn, Karl Jansen</x:v>
+        <x:v>Nozomu Kobayashi, Yoshiyuki Suimon, Koichi Miyamoto, Kosuke Mitarai</x:v>
       </x:c>
       <x:c r="E77" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00118-z</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00136-x</x:v>
       </x:c>
       <x:c r="F77" s="2" t="str">
         <x:v>QML</x:v>
@@ -2081,7 +2081,7 @@
     </x:row>
     <x:row r="78" ht="15.75">
       <x:c r="A78" s="2" t="str">
-        <x:v>Quantum Advantage Seeker with Kernels (QuASK): a software framework to speed up the research in quantum machine learning</x:v>
+        <x:v>A quantum “black box” for entropy calculation</x:v>
       </x:c>
       <x:c r="B78" s="2" t="n">
         <x:v>2023</x:v>
@@ -2090,10 +2090,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D78" s="2" t="str">
-        <x:v>Francesco Di Marcantonio, Massimiliano Incudini, Davide Tezza, Michele Grossi</x:v>
+        <x:v>Michal Koren, Oded Koren, Or Peretz</x:v>
       </x:c>
       <x:c r="E78" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00107-2</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00127-y</x:v>
       </x:c>
       <x:c r="F78" s="2" t="str">
         <x:v>QML</x:v>
@@ -2101,7 +2101,7 @@
     </x:row>
     <x:row r="79" ht="15.75">
       <x:c r="A79" s="2" t="str">
-        <x:v>Subtleties in the trainability of quantum machine learning models</x:v>
+        <x:v>Data re-uploading with a single qudit</x:v>
       </x:c>
       <x:c r="B79" s="2" t="n">
         <x:v>2023</x:v>
@@ -2110,10 +2110,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D79" s="2" t="str">
-        <x:v>Supanut Thanasilp, Samson Wang, Nhat Anh Nghiem, Patrick Coles, Marco Cerezo</x:v>
+        <x:v>Noah L. Wach, Manuel S. Rudolph, Fred Jendrzejewski, Sebastian Schmitt</x:v>
       </x:c>
       <x:c r="E79" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00103-6</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00125-0</x:v>
       </x:c>
       <x:c r="F79" s="2" t="str">
         <x:v>QML</x:v>
@@ -2121,7 +2121,7 @@
     </x:row>
     <x:row r="80" ht="15.75">
       <x:c r="A80" s="2" t="str">
-        <x:v>The effect of the processing and measurement operators on the expressive power of quantum models</x:v>
+        <x:v>Comparing quantum and classical machine learning for Vector Boson Scattering background reduction at the Large Hadron Collider</x:v>
       </x:c>
       <x:c r="B80" s="2" t="n">
         <x:v>2023</x:v>
@@ -2130,10 +2130,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D80" s="2" t="str">
-        <x:v>Aikaterini (Katerina) Gratsea, Patrick Huembeli </x:v>
+        <x:v>Davide Cugini, Dario Gerace, Pietro Govoni, Aurora Perego, Davide Valsecchi </x:v>
       </x:c>
       <x:c r="E80" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00109-0</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00106-3</x:v>
       </x:c>
       <x:c r="F80" s="2" t="str">
         <x:v>QML</x:v>
@@ -2141,7 +2141,7 @@
     </x:row>
     <x:row r="81" ht="15.75">
       <x:c r="A81" s="2" t="str">
-        <x:v>Estimating the degree of non-Markovianity using variational quantum circuits</x:v>
+        <x:v>Classical splitting of parametrized quantum circuits</x:v>
       </x:c>
       <x:c r="B81" s="2" t="n">
         <x:v>2023</x:v>
@@ -2150,10 +2150,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D81" s="2" t="str">
-        <x:v>Hossein T. Dinani, Diego Tancara, Felipe F. Fanchini, Ariel Norambuena, Raul Coto</x:v>
+        <x:v>Cenk Tüysüz, Giuseppe Clemente, Arianna Crippa, Tobias Hartung, Stefan Kühn, Karl Jansen</x:v>
       </x:c>
       <x:c r="E81" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00120-5</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00118-z</x:v>
       </x:c>
       <x:c r="F81" s="2" t="str">
         <x:v>QML</x:v>
@@ -2161,7 +2161,7 @@
     </x:row>
     <x:row r="82" ht="15.75">
       <x:c r="A82" s="2" t="str">
-        <x:v>Quantum Metropolis Solver: a quantum walks approach to optimization problems</x:v>
+        <x:v>Quantum Advantage Seeker with Kernels (QuASK): a software framework to speed up the research in quantum machine learning</x:v>
       </x:c>
       <x:c r="B82" s="2" t="n">
         <x:v>2023</x:v>
@@ -2170,10 +2170,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D82" s="2" t="str">
-        <x:v>Roberto Campos, P. A. M. Casares, M. A. Martin-Delgado</x:v>
+        <x:v>Francesco Di Marcantonio, Massimiliano Incudini, Davide Tezza, Michele Grossi</x:v>
       </x:c>
       <x:c r="E82" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00119-y</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00107-2</x:v>
       </x:c>
       <x:c r="F82" s="2" t="str">
         <x:v>QML</x:v>
@@ -2181,7 +2181,7 @@
     </x:row>
     <x:row r="83" ht="15.75">
       <x:c r="A83" s="2" t="str">
-        <x:v>Multi-level quantum inspired metaheuristics for automatic clustering of hyperspectral images</x:v>
+        <x:v>Subtleties in the trainability of quantum machine learning models</x:v>
       </x:c>
       <x:c r="B83" s="2" t="n">
         <x:v>2023</x:v>
@@ -2190,10 +2190,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D83" s="2" t="str">
-        <x:v>Tulika Dutta, Siddhartha Bhattacharyya, Bijaya Ketan Panigrahi, Ivan Zelinka &amp; Leo Mrsic </x:v>
+        <x:v>Supanut Thanasilp, Samson Wang, Nhat Anh Nghiem, Patrick Coles, Marco Cerezo</x:v>
       </x:c>
       <x:c r="E83" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00110-7</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00103-6</x:v>
       </x:c>
       <x:c r="F83" s="2" t="str">
         <x:v>QML</x:v>
@@ -2201,7 +2201,7 @@
     </x:row>
     <x:row r="84" ht="15.75">
       <x:c r="A84" s="2" t="str">
-        <x:v>MAQML: a Meta-approach to Quantum Machine Learning with Accentuated Sample Variations for Unobtrusive Mental Health Monitoring</x:v>
+        <x:v>The effect of the processing and measurement operators on the expressive power of quantum models</x:v>
       </x:c>
       <x:c r="B84" s="2" t="n">
         <x:v>2023</x:v>
@@ -2210,10 +2210,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D84" s="2" t="str">
-        <x:v>Anupama Padha &amp; Anita Sahoo </x:v>
+        <x:v>Aikaterini (Katerina) Gratsea, Patrick Huembeli </x:v>
       </x:c>
       <x:c r="E84" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00108-1</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00109-0</x:v>
       </x:c>
       <x:c r="F84" s="2" t="str">
         <x:v>QML</x:v>
@@ -2221,7 +2221,7 @@
     </x:row>
     <x:row r="85" ht="15.75">
       <x:c r="A85" s="2" t="str">
-        <x:v>Quantum pattern recognition on real quantum processing units</x:v>
+        <x:v>Estimating the degree of non-Markovianity using variational quantum circuits</x:v>
       </x:c>
       <x:c r="B85" s="2" t="n">
         <x:v>2023</x:v>
@@ -2230,10 +2230,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D85" s="2" t="str">
-        <x:v>Sreetama Das, Jingfu Zhang, Stefano Martina, Dieter Suter &amp; Filippo Caruso</x:v>
+        <x:v>Hossein T. Dinani, Diego Tancara, Felipe F. Fanchini, Ariel Norambuena, Raul Coto</x:v>
       </x:c>
       <x:c r="E85" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-022-00093-x</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00120-5</x:v>
       </x:c>
       <x:c r="F85" s="2" t="str">
         <x:v>QML</x:v>
@@ -2241,7 +2241,7 @@
     </x:row>
     <x:row r="86" ht="15.75">
       <x:c r="A86" s="2" t="str">
-        <x:v>If AI machine cannot think, can QI machine think?—from negative numbers to quantum intelligence for mind-light-matter unity</x:v>
+        <x:v>Quantum Metropolis Solver: a quantum walks approach to optimization problems</x:v>
       </x:c>
       <x:c r="B86" s="2" t="n">
         <x:v>2023</x:v>
@@ -2250,10 +2250,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D86" s="2" t="str">
-        <x:v>Wen-Ran Zhang </x:v>
+        <x:v>Roberto Campos, P. A. M. Casares, M. A. Martin-Delgado</x:v>
       </x:c>
       <x:c r="E86" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00104-5</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00119-y</x:v>
       </x:c>
       <x:c r="F86" s="2" t="str">
         <x:v>QML</x:v>
@@ -2261,19 +2261,19 @@
     </x:row>
     <x:row r="87" ht="15.75">
       <x:c r="A87" s="2" t="str">
-        <x:v>Converge of coordinate attention boosted YOLOv5 model and quantum dot labeled fluorescent biosensing for rapid detection of the poultry disease</x:v>
+        <x:v>Multi-level quantum inspired metaheuristics for automatic clustering of hyperspectral images</x:v>
       </x:c>
       <x:c r="B87" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C87" s="2" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D87" s="2" t="str">
-        <x:v>Yingchao Zhang, Hong Duan, Yuanjie Liu, Yanbin Li, Jianhan Lin</x:v>
+        <x:v>Tulika Dutta, Siddhartha Bhattacharyya, Bijaya Ketan Panigrahi, Ivan Zelinka &amp; Leo Mrsic </x:v>
       </x:c>
       <x:c r="E87" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.physleta.2023.129097</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00110-7</x:v>
       </x:c>
       <x:c r="F87" s="2" t="str">
         <x:v>QML</x:v>
@@ -2281,7 +2281,7 @@
     </x:row>
     <x:row r="88" ht="15.75">
       <x:c r="A88" s="2" t="str">
-        <x:v>Quantum Informed Machine-Learning Potentials for Molecular Dynamics Simulations of CO2’s Chemisorption and Diffusion in Mg-MOF-74</x:v>
+        <x:v>MAQML: a Meta-approach to Quantum Machine Learning with Accentuated Sample Variations for Unobtrusive Mental Health Monitoring</x:v>
       </x:c>
       <x:c r="B88" s="2" t="n">
         <x:v>2023</x:v>
@@ -2290,10 +2290,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D88" s="2" t="str">
-        <x:v>Bowen ZhengFelipe Lopes OliveiraRodrigo Neumann Barros FerreiraMathias SteinerHendrik HamannGrace X. GuBinquan Luan</x:v>
+        <x:v>Anupama Padha &amp; Anita Sahoo </x:v>
       </x:c>
       <x:c r="E88" s="2" t="str">
-        <x:v>https://doi.org/10.1021/acsnano.2c11102</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00108-1</x:v>
       </x:c>
       <x:c r="F88" s="2" t="str">
         <x:v>QML</x:v>
@@ -2301,7 +2301,7 @@
     </x:row>
     <x:row r="89" ht="15.75">
       <x:c r="A89" s="2" t="str">
-        <x:v>Efficient Quantum Algorithm for Nonlinear Reaction–Diffusion Equations and Energy Estimation</x:v>
+        <x:v>Quantum pattern recognition on real quantum processing units</x:v>
       </x:c>
       <x:c r="B89" s="2" t="n">
         <x:v>2023</x:v>
@@ -2310,10 +2310,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D89" s="2" t="str">
-        <x:v>Jin-Peng Liu, Dong An, Di Fang, Jiasu Wang, Guang Hao Low &amp; Stephen Jordan</x:v>
+        <x:v>Sreetama Das, Jingfu Zhang, Stefano Martina, Dieter Suter &amp; Filippo Caruso</x:v>
       </x:c>
       <x:c r="E89" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s00220-023-04857-9</x:v>
+        <x:v>https://doi.org/10.1007/s42484-022-00093-x</x:v>
       </x:c>
       <x:c r="F89" s="2" t="str">
         <x:v>QML</x:v>
@@ -2321,19 +2321,19 @@
     </x:row>
     <x:row r="90" ht="15.75">
       <x:c r="A90" s="2" t="str">
-        <x:v>Optimizing Quantum Classification Algorithms on Classical Benchmark Datasets</x:v>
+        <x:v>If AI machine cannot think, can QI machine think?—from negative numbers to quantum intelligence for mind-light-matter unity</x:v>
       </x:c>
       <x:c r="B90" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C90" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D90" s="2" t="str">
-        <x:v>Manuel John ,Julian Schuhmacher, Panagiotis Barkoutsos, vano Tavernelli and Francesco Tacchino</x:v>
+        <x:v>Wen-Ran Zhang </x:v>
       </x:c>
       <x:c r="E90" s="2" t="str">
-        <x:v>https://doi.org/10.3390/e25060860</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00104-5</x:v>
       </x:c>
       <x:c r="F90" s="2" t="str">
         <x:v>QML</x:v>
@@ -2341,19 +2341,19 @@
     </x:row>
     <x:row r="91" ht="15.75">
       <x:c r="A91" s="2" t="str">
-        <x:v>An Enhanced Quantum K-Nearest Neighbor Classification Algorithm Based on Polar Distance</x:v>
+        <x:v>Converge of coordinate attention boosted YOLOv5 model and quantum dot labeled fluorescent biosensing for rapid detection of the poultry disease</x:v>
       </x:c>
       <x:c r="B91" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C91" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D91" s="2" t="str">
-        <x:v>Congcong Feng ,Bo Zhao,Xin Zhou,Xiaodong Ding and Zheng Shan </x:v>
+        <x:v>Yingchao Zhang, Hong Duan, Yuanjie Liu, Yanbin Li, Jianhan Lin</x:v>
       </x:c>
       <x:c r="E91" s="2" t="str">
-        <x:v>https://doi.org/10.3390/e25010127</x:v>
+        <x:v>https://doi.org/10.1016/j.physleta.2023.129097</x:v>
       </x:c>
       <x:c r="F91" s="2" t="str">
         <x:v>QML</x:v>
@@ -2361,19 +2361,19 @@
     </x:row>
     <x:row r="92" ht="15.75">
       <x:c r="A92" s="2" t="str">
-        <x:v>Quantum Machine Learning—An Overview</x:v>
+        <x:v>Quantum Informed Machine-Learning Potentials for Molecular Dynamics Simulations of CO2’s Chemisorption and Diffusion in Mg-MOF-74</x:v>
       </x:c>
       <x:c r="B92" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C92" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D92" s="2" t="str">
-        <x:v> Kyriaki A. Tychola,Theofanis Kalampokas and George A. Papakostas</x:v>
+        <x:v>Bowen ZhengFelipe Lopes OliveiraRodrigo Neumann Barros FerreiraMathias SteinerHendrik HamannGrace X. GuBinquan Luan</x:v>
       </x:c>
       <x:c r="E92" s="2" t="str">
-        <x:v>https://doi.org/10.3390/electronics12112379</x:v>
+        <x:v>https://doi.org/10.1021/acsnano.2c11102</x:v>
       </x:c>
       <x:c r="F92" s="2" t="str">
         <x:v>QML</x:v>
@@ -2381,19 +2381,19 @@
     </x:row>
     <x:row r="93" ht="15.75">
       <x:c r="A93" s="2" t="str">
-        <x:v>Performance Evaluation of Quantum-Based Machine Learning Algorithms for Cardiac Arrhythmia Classification</x:v>
+        <x:v>Efficient Quantum Algorithm for Nonlinear Reaction–Diffusion Equations and Energy Estimation</x:v>
       </x:c>
       <x:c r="B93" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C93" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D93" s="2" t="str">
-        <x:v>Zeynep Ozpolat and Murat Karabatak </x:v>
+        <x:v>Jin-Peng Liu, Dong An, Di Fang, Jiasu Wang, Guang Hao Low &amp; Stephen Jordan</x:v>
       </x:c>
       <x:c r="E93" s="2" t="str">
-        <x:v>https://doi.org/10.3390/diagnostics13061099</x:v>
+        <x:v>https://doi.org/10.1007/s00220-023-04857-9</x:v>
       </x:c>
       <x:c r="F93" s="2" t="str">
         <x:v>QML</x:v>
@@ -2401,19 +2401,19 @@
     </x:row>
     <x:row r="94" ht="15.75">
       <x:c r="A94" s="2" t="str">
-        <x:v>Quantum Machine Learning: A tutorial</x:v>
+        <x:v>Optimizing Quantum Classification Algorithms on Classical Benchmark Datasets</x:v>
       </x:c>
       <x:c r="B94" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C94" s="2" t="str">
-        <x:v>Neurocomputing</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D94" s="2" t="str">
-        <x:v>José D. Martín-Guerrero a, Lucas Lamata</x:v>
+        <x:v>Manuel John ,Julian Schuhmacher, Panagiotis Barkoutsos, vano Tavernelli and Francesco Tacchino</x:v>
       </x:c>
       <x:c r="E94" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/pii/S0925231221011000</x:v>
+        <x:v>https://doi.org/10.3390/e25060860</x:v>
       </x:c>
       <x:c r="F94" s="2" t="str">
         <x:v>QML</x:v>
@@ -2421,19 +2421,19 @@
     </x:row>
     <x:row r="95" ht="15.75">
       <x:c r="A95" s="2" t="str">
-        <x:v>Challenges and opportunities in quantum machine learning</x:v>
+        <x:v>An Enhanced Quantum K-Nearest Neighbor Classification Algorithm Based on Polar Distance</x:v>
       </x:c>
       <x:c r="B95" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C95" s="2" t="str">
-        <x:v>nature computational science</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D95" s="2" t="str">
-        <x:v>    M. Cerezo, Guillaume Verdon, Hsin-Yuan Huang, Lukasz Cincio &amp; Patrick J. Coles</x:v>
+        <x:v>Congcong Feng ,Bo Zhao,Xin Zhou,Xiaodong Ding and Zheng Shan </x:v>
       </x:c>
       <x:c r="E95" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s43588-022-00311-3</x:v>
+        <x:v>https://doi.org/10.3390/e25010127</x:v>
       </x:c>
       <x:c r="F95" s="2" t="str">
         <x:v>QML</x:v>
@@ -2441,19 +2441,19 @@
     </x:row>
     <x:row r="96" ht="15.75">
       <x:c r="A96" s="2" t="str">
-        <x:v>Is Quantum Advantage the Right Goal for Quantum Machine Learning?</x:v>
+        <x:v>Quantum Machine Learning—An Overview</x:v>
       </x:c>
       <x:c r="B96" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C96" s="2" t="str">
-        <x:v>PRX Quantum 3</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D96" s="2" t="str">
-        <x:v>Maria Schuld and Nathan Killoran</x:v>
+        <x:v> Kyriaki A. Tychola,Theofanis Kalampokas and George A. Papakostas</x:v>
       </x:c>
       <x:c r="E96" s="2" t="str">
-        <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.3.030101</x:v>
+        <x:v>https://doi.org/10.3390/electronics12112379</x:v>
       </x:c>
       <x:c r="F96" s="2" t="str">
         <x:v>QML</x:v>
@@ -2461,19 +2461,19 @@
     </x:row>
     <x:row r="97" ht="15.75">
       <x:c r="A97" s="2" t="str">
-        <x:v>Quantum machine learning for chemistry and physics</x:v>
+        <x:v>Performance Evaluation of Quantum-Based Machine Learning Algorithms for Cardiac Arrhythmia Classification</x:v>
       </x:c>
       <x:c r="B97" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C97" s="2" t="str">
-        <x:v>Chem. Soc. Rev</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D97" s="2" t="str">
-        <x:v>Manas Sajjan , Junxu Li</x:v>
+        <x:v>Zeynep Ozpolat and Murat Karabatak </x:v>
       </x:c>
       <x:c r="E97" s="2" t="str">
-        <x:v>https://pubs.rsc.org/en/content/articlehtml/2022/cs/d2cs00203e</x:v>
+        <x:v>https://doi.org/10.3390/diagnostics13061099</x:v>
       </x:c>
       <x:c r="F97" s="2" t="str">
         <x:v>QML</x:v>
@@ -2481,19 +2481,19 @@
     </x:row>
     <x:row r="98" ht="15.75">
       <x:c r="A98" s="2" t="str">
-        <x:v>Generalization in quantum machine learning from few training data</x:v>
+        <x:v>Quantum Machine Learning: A tutorial</x:v>
       </x:c>
       <x:c r="B98" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C98" s="2" t="str">
-        <x:v>nature communications</x:v>
+        <x:v>Neurocomputing</x:v>
       </x:c>
       <x:c r="D98" s="2" t="str">
-        <x:v>Matthias C. Caro, Hsin-Yuan Huang, M. Cerezo, Kunal Sharma, Andrew Sornborger, Lukasz Cincio &amp; Patrick J. Coles</x:v>
+        <x:v>José D. Martín-Guerrero a, Lucas Lamata</x:v>
       </x:c>
       <x:c r="E98" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s41467-022-32550-3</x:v>
+        <x:v>https://www.sciencedirect.com/science/article/pii/S0925231221011000</x:v>
       </x:c>
       <x:c r="F98" s="2" t="str">
         <x:v>QML</x:v>
@@ -2501,19 +2501,19 @@
     </x:row>
     <x:row r="99" ht="15.75">
       <x:c r="A99" s="2" t="str">
-        <x:v>Group-Invariant Quantum Machine Learning</x:v>
+        <x:v>Challenges and opportunities in quantum machine learning</x:v>
       </x:c>
       <x:c r="B99" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C99" s="2" t="str">
-        <x:v>PRX Quantum</x:v>
+        <x:v>nature computational science</x:v>
       </x:c>
       <x:c r="D99" s="2" t="str">
-        <x:v>Martín Larocca, Frédéric Sauvage, Faris M. Sbahi, Guillaume Verdon, Patrick J. Coles, and M. Cerezo</x:v>
+        <x:v>    M. Cerezo, Guillaume Verdon, Hsin-Yuan Huang, Lukasz Cincio &amp; Patrick J. Coles</x:v>
       </x:c>
       <x:c r="E99" s="2" t="str">
-        <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.3.030341</x:v>
+        <x:v>https://www.nature.com/articles/s43588-022-00311-3</x:v>
       </x:c>
       <x:c r="F99" s="2" t="str">
         <x:v>QML</x:v>
@@ -2521,19 +2521,19 @@
     </x:row>
     <x:row r="100" ht="15.75">
       <x:c r="A100" s="2" t="str">
-        <x:v>An Introduction to Quantum Machine Learning for Engineers</x:v>
+        <x:v>Is Quantum Advantage the Right Goal for Quantum Machine Learning?</x:v>
       </x:c>
       <x:c r="B100" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C100" s="2" t="str">
-        <x:v>Foundations and Trends® in Signal Processing</x:v>
+        <x:v>PRX Quantum 3</x:v>
       </x:c>
       <x:c r="D100" s="2" t="str">
-        <x:v>Osvaldo Simeone</x:v>
+        <x:v>Maria Schuld and Nathan Killoran</x:v>
       </x:c>
       <x:c r="E100" s="2" t="str">
-        <x:v>https://www.nowpublishers.com/article/Details/SIG-118</x:v>
+        <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.3.030101</x:v>
       </x:c>
       <x:c r="F100" s="2" t="str">
         <x:v>QML</x:v>
@@ -2541,19 +2541,19 @@
     </x:row>
     <x:row r="101" ht="15.75">
       <x:c r="A101" s="2" t="str">
-        <x:v>Data compression for quantum machine learning</x:v>
+        <x:v>Quantum machine learning for chemistry and physics</x:v>
       </x:c>
       <x:c r="B101" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C101" s="2" t="str">
-        <x:v>Phys. Rev. Research 4</x:v>
+        <x:v>Chem. Soc. Rev</x:v>
       </x:c>
       <x:c r="D101" s="2" t="str">
-        <x:v>Rohit Dilip, Yu-Jie Liu, Adam Smith, and Frank Pollmann</x:v>
+        <x:v>Manas Sajjan , Junxu Li</x:v>
       </x:c>
       <x:c r="E101" s="2" t="str">
-        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.043007</x:v>
+        <x:v>https://pubs.rsc.org/en/content/articlehtml/2022/cs/d2cs00203e</x:v>
       </x:c>
       <x:c r="F101" s="2" t="str">
         <x:v>QML</x:v>
@@ -2561,19 +2561,19 @@
     </x:row>
     <x:row r="102" ht="15.75">
       <x:c r="A102" s="2" t="str">
-        <x:v>Representation Theory for Geometric Quantum Machine Learning</x:v>
+        <x:v>Generalization in quantum machine learning from few training data</x:v>
       </x:c>
       <x:c r="B102" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C102" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>nature communications</x:v>
       </x:c>
       <x:c r="D102" s="2" t="str">
-        <x:v>Michael Ragone, Paolo Braccia, Quynh T. Nguyen, Louis Schatzki, Patrick J. Coles, Frederic Sauvage, Martin Larocca, M. Cerezo</x:v>
+        <x:v>Matthias C. Caro, Hsin-Yuan Huang, M. Cerezo, Kunal Sharma, Andrew Sornborger, Lukasz Cincio &amp; Patrick J. Coles</x:v>
       </x:c>
       <x:c r="E102" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2210.07980</x:v>
+        <x:v>https://www.nature.com/articles/s41467-022-32550-3</x:v>
       </x:c>
       <x:c r="F102" s="2" t="str">
         <x:v>QML</x:v>
@@ -2581,19 +2581,19 @@
     </x:row>
     <x:row r="103" ht="15.75">
       <x:c r="A103" s="2" t="str">
-        <x:v>Importance of kernel bandwidth in quantum machine learning</x:v>
+        <x:v>Group-Invariant Quantum Machine Learning</x:v>
       </x:c>
       <x:c r="B103" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C103" s="2" t="str">
-        <x:v>Phys. Rev. A 106</x:v>
+        <x:v>PRX Quantum</x:v>
       </x:c>
       <x:c r="D103" s="2" t="str">
-        <x:v>Ruslan Shaydulin and Stefan M. Wild</x:v>
+        <x:v>Martín Larocca, Frédéric Sauvage, Faris M. Sbahi, Guillaume Verdon, Patrick J. Coles, and M. Cerezo</x:v>
       </x:c>
       <x:c r="E103" s="2" t="str">
-        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.106.042407</x:v>
+        <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.3.030341</x:v>
       </x:c>
       <x:c r="F103" s="2" t="str">
         <x:v>QML</x:v>
@@ -2601,19 +2601,19 @@
     </x:row>
     <x:row r="104" ht="15.75">
       <x:c r="A104" s="2" t="str">
-        <x:v>The Development of Quantum Machine Learning</x:v>
+        <x:v>An Introduction to Quantum Machine Learning for Engineers</x:v>
       </x:c>
       <x:c r="B104" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C104" s="2" t="str">
-        <x:v>Harvard Data Science Review</x:v>
+        <x:v>Foundations and Trends® in Signal Processing</x:v>
       </x:c>
       <x:c r="D104" s="2" t="str">
-        <x:v>Khadijeh Najafi</x:v>
+        <x:v>Osvaldo Simeone</x:v>
       </x:c>
       <x:c r="E104" s="2" t="str">
-        <x:v>https://assets.pubpub.org/05lwd2lr/5a9fd72c-212a-4a7d-91ba-07219d24359d.pdf</x:v>
+        <x:v>https://www.nowpublishers.com/article/Details/SIG-118</x:v>
       </x:c>
       <x:c r="F104" s="2" t="str">
         <x:v>QML</x:v>
@@ -2621,19 +2621,19 @@
     </x:row>
     <x:row r="105" ht="15.75">
       <x:c r="A105" s="2" t="str">
-        <x:v>Quantum Machine Learning Applications in the Biomedical Domain: A Systematic Review</x:v>
+        <x:v>Data compression for quantum machine learning</x:v>
       </x:c>
       <x:c r="B105" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C105" s="2" t="str">
-        <x:v>IEEE Access</x:v>
+        <x:v>Phys. Rev. Research 4</x:v>
       </x:c>
       <x:c r="D105" s="2" t="str">
-        <x:v>Danyal Maheshwari; Begonya Garcia-Zapirain; Daniel Sierra-Sosa</x:v>
+        <x:v>Rohit Dilip, Yu-Jie Liu, Adam Smith, and Frank Pollmann</x:v>
       </x:c>
       <x:c r="E105" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9844718</x:v>
+        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.043007</x:v>
       </x:c>
       <x:c r="F105" s="2" t="str">
         <x:v>QML</x:v>
@@ -2641,19 +2641,19 @@
     </x:row>
     <x:row r="106" ht="15.75">
       <x:c r="A106" s="2" t="str">
-        <x:v>Quantum machine-learning for medicinal chemistry</x:v>
+        <x:v>Representation Theory for Geometric Quantum Machine Learning</x:v>
       </x:c>
       <x:c r="B106" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C106" s="2" t="str">
-        <x:v>Phys. Chem. Chem. Phys</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D106" s="2" t="str">
-        <x:v>Kenneth Atz, Clemens Isert, Markus N. A. Böcker, José Jiménez-Luna and Gisbert Schneider</x:v>
+        <x:v>Michael Ragone, Paolo Braccia, Quynh T. Nguyen, Louis Schatzki, Patrick J. Coles, Frederic Sauvage, Martin Larocca, M. Cerezo</x:v>
       </x:c>
       <x:c r="E106" s="2" t="str">
-        <x:v>https://pubs.rsc.org/en/content/articlehtml/2022/cp/d2cp00834c</x:v>
+        <x:v>https://arxiv.org/abs/2210.07980</x:v>
       </x:c>
       <x:c r="F106" s="2" t="str">
         <x:v>QML</x:v>
@@ -2661,19 +2661,19 @@
     </x:row>
     <x:row r="107" ht="15.75">
       <x:c r="A107" s="2" t="str">
-        <x:v>Quantum Embedding Search for Quantum Machine Learning</x:v>
+        <x:v>Importance of kernel bandwidth in quantum machine learning</x:v>
       </x:c>
       <x:c r="B107" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C107" s="2" t="str">
-        <x:v>IEEE Access</x:v>
+        <x:v>Phys. Rev. A 106</x:v>
       </x:c>
       <x:c r="D107" s="2" t="str">
-        <x:v>Nam Nguyen; Kwang-Cheng Chen</x:v>
+        <x:v>Ruslan Shaydulin and Stefan M. Wild</x:v>
       </x:c>
       <x:c r="E107" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9757160</x:v>
+        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.106.042407</x:v>
       </x:c>
       <x:c r="F107" s="2" t="str">
         <x:v>QML</x:v>
@@ -2681,19 +2681,19 @@
     </x:row>
     <x:row r="108" ht="15.75">
       <x:c r="A108" s="2" t="str">
-        <x:v>Quantum machine learning with subspace states</x:v>
+        <x:v>The Development of Quantum Machine Learning</x:v>
       </x:c>
       <x:c r="B108" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C108" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Harvard Data Science Review</x:v>
       </x:c>
       <x:c r="D108" s="2" t="str">
-        <x:v>Iordanis Kerenidis, Anupam Prakash</x:v>
+        <x:v>Khadijeh Najafi</x:v>
       </x:c>
       <x:c r="E108" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2202.00054</x:v>
+        <x:v>https://assets.pubpub.org/05lwd2lr/5a9fd72c-212a-4a7d-91ba-07219d24359d.pdf</x:v>
       </x:c>
       <x:c r="F108" s="2" t="str">
         <x:v>QML</x:v>
@@ -2701,19 +2701,19 @@
     </x:row>
     <x:row r="109" ht="15.75">
       <x:c r="A109" s="2" t="str">
-        <x:v>Quantum Machine Learning for b-jet charge identification</x:v>
+        <x:v>Quantum Machine Learning Applications in the Biomedical Domain: A Systematic Review</x:v>
       </x:c>
       <x:c r="B109" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C109" s="2" t="str">
-        <x:v>Journal of High Energy Physics</x:v>
+        <x:v>IEEE Access</x:v>
       </x:c>
       <x:c r="D109" s="2" t="str">
-        <x:v>Alessio Gianelle, Patrick Koppenburg, Donatella Lucchesi, Davide Nicotra, Eduardo Rodrigues, Lorenzo Sestini, Jacco de Vries &amp; Davide Zuliani</x:v>
+        <x:v>Danyal Maheshwari; Begonya Garcia-Zapirain; Daniel Sierra-Sosa</x:v>
       </x:c>
       <x:c r="E109" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/JHEP08(2022)014</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9844718</x:v>
       </x:c>
       <x:c r="F109" s="2" t="str">
         <x:v>QML</x:v>
@@ -2721,19 +2721,19 @@
     </x:row>
     <x:row r="110" ht="15.75">
       <x:c r="A110" s="2" t="str">
-        <x:v>A Comprehensive Survey on Quantum Machine Learning and Possible Applications</x:v>
+        <x:v>Quantum machine-learning for medicinal chemistry</x:v>
       </x:c>
       <x:c r="B110" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C110" s="2" t="str">
-        <x:v>International Journal of E-Health and Medical Communications (IJEHMC) </x:v>
+        <x:v>Phys. Chem. Chem. Phys</x:v>
       </x:c>
       <x:c r="D110" s="2" t="str">
-        <x:v>Muhammad Junaid Umer, Muhammad Imran Sharif</x:v>
+        <x:v>Kenneth Atz, Clemens Isert, Markus N. A. Böcker, José Jiménez-Luna and Gisbert Schneider</x:v>
       </x:c>
       <x:c r="E110" s="2" t="str">
-        <x:v>https://www.igi-global.com/article/a-comprehensive-survey-on-quantum-machine-learning-and-possible-applications/315730</x:v>
+        <x:v>https://pubs.rsc.org/en/content/articlehtml/2022/cp/d2cp00834c</x:v>
       </x:c>
       <x:c r="F110" s="2" t="str">
         <x:v>QML</x:v>
@@ -2741,19 +2741,19 @@
     </x:row>
     <x:row r="111" ht="15.75">
       <x:c r="A111" s="2" t="str">
-        <x:v>Comparative performance analysis of quantum machine learning with deep learning for diabetes prediction</x:v>
+        <x:v>Quantum Embedding Search for Quantum Machine Learning</x:v>
       </x:c>
       <x:c r="B111" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C111" s="2" t="str">
-        <x:v>Complex &amp; Intelligent Systems</x:v>
+        <x:v>IEEE Access</x:v>
       </x:c>
       <x:c r="D111" s="2" t="str">
-        <x:v>Himanshu Gupta, Hirdesh Varshney, Tarun Kumar Sharma, Nikhil Pachauri &amp; Om Prakash Verma</x:v>
+        <x:v>Nam Nguyen; Kwang-Cheng Chen</x:v>
       </x:c>
       <x:c r="E111" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s40747-021-00398-7</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9757160</x:v>
       </x:c>
       <x:c r="F111" s="2" t="str">
         <x:v>QML</x:v>
@@ -2761,19 +2761,19 @@
     </x:row>
     <x:row r="112" ht="15.75">
       <x:c r="A112" s="2" t="str">
-        <x:v>Machine learning in the quantum realm: The state-of-the-art, challenges, and future vision</x:v>
+        <x:v>Quantum machine learning with subspace states</x:v>
       </x:c>
       <x:c r="B112" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C112" s="2" t="str">
-        <x:v>Expert Systems with Applications</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D112" s="2" t="str">
-        <x:v>Essam H. Houssein a, Zainab Abohashima b, Mohamed Elhoseny c d, Waleed M. Mohamed</x:v>
+        <x:v>Iordanis Kerenidis, Anupam Prakash</x:v>
       </x:c>
       <x:c r="E112" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0957417422000136</x:v>
+        <x:v>https://arxiv.org/abs/2202.00054</x:v>
       </x:c>
       <x:c r="F112" s="2" t="str">
         <x:v>QML</x:v>
@@ -2781,19 +2781,19 @@
     </x:row>
     <x:row r="113" ht="15.75">
       <x:c r="A113" s="2" t="str">
-        <x:v>Quantum-machine-learning channel discrimination</x:v>
+        <x:v>Quantum Machine Learning for b-jet charge identification</x:v>
       </x:c>
       <x:c r="B113" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C113" s="2" t="str">
-        <x:v>Phys. Rev. A 106</x:v>
+        <x:v>Journal of High Energy Physics</x:v>
       </x:c>
       <x:c r="D113" s="2" t="str">
-        <x:v>A. S. Kardashin, A. V. Vlasova, A. A. Pervishko, D. Yudin, and J. D. Biamonte</x:v>
+        <x:v>Alessio Gianelle, Patrick Koppenburg, Donatella Lucchesi, Davide Nicotra, Eduardo Rodrigues, Lorenzo Sestini, Jacco de Vries &amp; Davide Zuliani</x:v>
       </x:c>
       <x:c r="E113" s="2" t="str">
-        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.106.032409</x:v>
+        <x:v>https://link.springer.com/article/10.1007/JHEP08(2022)014</x:v>
       </x:c>
       <x:c r="F113" s="2" t="str">
         <x:v>QML</x:v>
@@ -2801,19 +2801,19 @@
     </x:row>
     <x:row r="114" ht="15.75">
       <x:c r="A114" s="2" t="str">
-        <x:v>BIGDML—Towards accurate quantum machine learning force fields for materials</x:v>
+        <x:v>A Comprehensive Survey on Quantum Machine Learning and Possible Applications</x:v>
       </x:c>
       <x:c r="B114" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C114" s="2" t="str">
-        <x:v>nature communications</x:v>
+        <x:v>International Journal of E-Health and Medical Communications (IJEHMC) </x:v>
       </x:c>
       <x:c r="D114" s="2" t="str">
-        <x:v>Huziel E. Sauceda, Luis E. Gálvez-González, Stefan Chmiela, Lauro Oliver Paz-Borbón, Klaus-Robert Müller &amp; Alexandre Tkatchenko</x:v>
+        <x:v>Muhammad Junaid Umer, Muhammad Imran Sharif</x:v>
       </x:c>
       <x:c r="E114" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s41467-022-31093-x</x:v>
+        <x:v>https://www.igi-global.com/article/a-comprehensive-survey-on-quantum-machine-learning-and-possible-applications/315730</x:v>
       </x:c>
       <x:c r="F114" s="2" t="str">
         <x:v>QML</x:v>
@@ -2821,19 +2821,19 @@
     </x:row>
     <x:row r="115" ht="15.75">
       <x:c r="A115" s="2" t="str">
-        <x:v>Quantum Machine Learning in Finance: Time Series Forecasting</x:v>
+        <x:v>Comparative performance analysis of quantum machine learning with deep learning for diabetes prediction</x:v>
       </x:c>
       <x:c r="B115" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C115" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Complex &amp; Intelligent Systems</x:v>
       </x:c>
       <x:c r="D115" s="2" t="str">
-        <x:v>Dimitrios Emmanoulopoulos, Sofija Dimoska</x:v>
+        <x:v>Himanshu Gupta, Hirdesh Varshney, Tarun Kumar Sharma, Nikhil Pachauri &amp; Om Prakash Verma</x:v>
       </x:c>
       <x:c r="E115" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2202.00599</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s40747-021-00398-7</x:v>
       </x:c>
       <x:c r="F115" s="2" t="str">
         <x:v>QML</x:v>
@@ -2841,19 +2841,19 @@
     </x:row>
     <x:row r="116" ht="15.75">
       <x:c r="A116" s="2" t="str">
-        <x:v>On establishing learning separations between classical and quantum machine learning with classical data</x:v>
+        <x:v>Machine learning in the quantum realm: The state-of-the-art, challenges, and future vision</x:v>
       </x:c>
       <x:c r="B116" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C116" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Expert Systems with Applications</x:v>
       </x:c>
       <x:c r="D116" s="2" t="str">
-        <x:v>Casper Gyurik, Vedran Dunjko</x:v>
+        <x:v>Essam H. Houssein a, Zainab Abohashima b, Mohamed Elhoseny c d, Waleed M. Mohamed</x:v>
       </x:c>
       <x:c r="E116" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2208.06339</x:v>
+        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0957417422000136</x:v>
       </x:c>
       <x:c r="F116" s="2" t="str">
         <x:v>QML</x:v>
@@ -2861,19 +2861,19 @@
     </x:row>
     <x:row r="117" ht="15.75">
       <x:c r="A117" s="2" t="str">
-        <x:v>Qsun: an open-source platform towards practical quantum machine learning applications</x:v>
+        <x:v>Quantum-machine-learning channel discrimination</x:v>
       </x:c>
       <x:c r="B117" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C117" s="2" t="str">
-        <x:v>Machine Learning: Science and Technology</x:v>
+        <x:v>Phys. Rev. A 106</x:v>
       </x:c>
       <x:c r="D117" s="2" t="str">
-        <x:v>Quoc Chuong Nguyen5,1, Le Bin Ho, Lan Nguyen Tran2 and Hung Q Nguyen</x:v>
+        <x:v>A. S. Kardashin, A. V. Vlasova, A. A. Pervishko, D. Yudin, and J. D. Biamonte</x:v>
       </x:c>
       <x:c r="E117" s="2" t="str">
-        <x:v>https://iopscience.iop.org/article/10.1088/2632-2153/ac5997/meta</x:v>
+        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.106.032409</x:v>
       </x:c>
       <x:c r="F117" s="2" t="str">
         <x:v>QML</x:v>
@@ -2881,19 +2881,19 @@
     </x:row>
     <x:row r="118" ht="15.75">
       <x:c r="A118" s="2" t="str">
-        <x:v>Challenges and opportunities in quantum machine learning for high-energy physics</x:v>
+        <x:v>BIGDML—Towards accurate quantum machine learning force fields for materials</x:v>
       </x:c>
       <x:c r="B118" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C118" s="2" t="str">
-        <x:v>Nature Reviews Physics</x:v>
+        <x:v>nature communications</x:v>
       </x:c>
       <x:c r="D118" s="2" t="str">
-        <x:v>Sau Lan Wu &amp; Shinjae Yoo</x:v>
+        <x:v>Huziel E. Sauceda, Luis E. Gálvez-González, Stefan Chmiela, Lauro Oliver Paz-Borbón, Klaus-Robert Müller &amp; Alexandre Tkatchenko</x:v>
       </x:c>
       <x:c r="E118" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s42254-022-00425-7</x:v>
+        <x:v>https://www.nature.com/articles/s41467-022-31093-x</x:v>
       </x:c>
       <x:c r="F118" s="2" t="str">
         <x:v>QML</x:v>
@@ -2901,19 +2901,19 @@
     </x:row>
     <x:row r="119" ht="15.75">
       <x:c r="A119" s="2" t="str">
-        <x:v>Retrieving information from a black hole using quantum machine learning</x:v>
+        <x:v>Quantum Machine Learning in Finance: Time Series Forecasting</x:v>
       </x:c>
       <x:c r="B119" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C119" s="2" t="str">
-        <x:v>Phys. Rev. A 106</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D119" s="2" t="str">
-        <x:v>Lorenzo Leone, Salvatore F. E. Oliviero, Stefano Piemontese, Sarah True, and Alioscia Hamma</x:v>
+        <x:v>Dimitrios Emmanoulopoulos, Sofija Dimoska</x:v>
       </x:c>
       <x:c r="E119" s="2" t="str">
-        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.106.062434</x:v>
+        <x:v>https://arxiv.org/abs/2202.00599</x:v>
       </x:c>
       <x:c r="F119" s="2" t="str">
         <x:v>QML</x:v>
@@ -2921,19 +2921,19 @@
     </x:row>
     <x:row r="120" ht="15.75">
       <x:c r="A120" s="2" t="str">
-        <x:v>Matrix product state pre-training for quantum machine learning</x:v>
+        <x:v>On establishing learning separations between classical and quantum machine learning with classical data</x:v>
       </x:c>
       <x:c r="B120" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C120" s="2" t="str">
-        <x:v>Quantum Science and Technology</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D120" s="2" t="str">
-        <x:v>James Dborin, Fergus Barratt, Vinul Wimalaweera, Lewis Wright and Andrew G Green</x:v>
+        <x:v>Casper Gyurik, Vedran Dunjko</x:v>
       </x:c>
       <x:c r="E120" s="2" t="str">
-        <x:v>https://iopscience.iop.org/article/10.1088/2058-9565/ac7073/meta</x:v>
+        <x:v>https://arxiv.org/abs/2208.06339</x:v>
       </x:c>
       <x:c r="F120" s="2" t="str">
         <x:v>QML</x:v>
@@ -2941,19 +2941,19 @@
     </x:row>
     <x:row r="121" ht="15.75">
       <x:c r="A121" s="2" t="str">
-        <x:v>An orbital-based representation for accurate quantum machine learning </x:v>
+        <x:v>Qsun: an open-source platform towards practical quantum machine learning applications</x:v>
       </x:c>
       <x:c r="B121" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C121" s="2" t="str">
-        <x:v>The Journal of Chemical Physics</x:v>
+        <x:v>Machine Learning: Science and Technology</x:v>
       </x:c>
       <x:c r="D121" s="2" t="str">
-        <x:v>Konstantin Karandashev; O. Anatole von Lilienfeld</x:v>
+        <x:v>Quoc Chuong Nguyen5,1, Le Bin Ho, Lan Nguyen Tran2 and Hung Q Nguyen</x:v>
       </x:c>
       <x:c r="E121" s="2" t="str">
-        <x:v>https://pubs.aip.org/aip/jcp/article-abstract/156/11/114101/2840879/An-orbital-based-representation-for-accurate?redirectedFrom=fulltext</x:v>
+        <x:v>https://iopscience.iop.org/article/10.1088/2632-2153/ac5997/meta</x:v>
       </x:c>
       <x:c r="F121" s="2" t="str">
         <x:v>QML</x:v>
@@ -2961,19 +2961,19 @@
     </x:row>
     <x:row r="122" ht="15.75">
       <x:c r="A122" s="2" t="str">
-        <x:v>Quantum Machine Learning Approach for Studying Atmospheric Cluster Formation</x:v>
+        <x:v>Challenges and opportunities in quantum machine learning for high-energy physics</x:v>
       </x:c>
       <x:c r="B122" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C122" s="2" t="str">
-        <x:v>Environmental Science &amp; Technology Letters</x:v>
+        <x:v>Nature Reviews Physics</x:v>
       </x:c>
       <x:c r="D122" s="2" t="str">
-        <x:v>Jakub Kubečka, Anders S. Christensen, Freja Rydahl Rasmussen,, Jonas Elm</x:v>
+        <x:v>Sau Lan Wu &amp; Shinjae Yoo</x:v>
       </x:c>
       <x:c r="E122" s="2" t="str">
-        <x:v>https://pubs.acs.org/doi/abs/10.1021/acs.estlett.1c00997</x:v>
+        <x:v>https://www.nature.com/articles/s42254-022-00425-7</x:v>
       </x:c>
       <x:c r="F122" s="2" t="str">
         <x:v>QML</x:v>
@@ -2981,19 +2981,19 @@
     </x:row>
     <x:row r="123" ht="15.75">
       <x:c r="A123" s="2" t="str">
-        <x:v>Overfitting in quantum machine learning and entangling dropout</x:v>
+        <x:v>Retrieving information from a black hole using quantum machine learning</x:v>
       </x:c>
       <x:c r="B123" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C123" s="2" t="str">
-        <x:v>Quantum Machine Intelligence</x:v>
+        <x:v>Phys. Rev. A 106</x:v>
       </x:c>
       <x:c r="D123" s="2" t="str">
-        <x:v>Masahiro Kobayashi, Kouhei Nakaji &amp; Naoki Yamamoto</x:v>
+        <x:v>Lorenzo Leone, Salvatore F. E. Oliviero, Stefano Piemontese, Sarah True, and Alioscia Hamma</x:v>
       </x:c>
       <x:c r="E123" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s42484-022-00087-9</x:v>
+        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.106.062434</x:v>
       </x:c>
       <x:c r="F123" s="2" t="str">
         <x:v>QML</x:v>
@@ -3001,19 +3001,19 @@
     </x:row>
     <x:row r="124">
       <x:c r="A124" s="2" t="str">
-        <x:v>Sampling-based Sublinear Low-rank Matrix Arithmetic Framework for Dequantizing Quantum Machine Learning</x:v>
+        <x:v>Matrix product state pre-training for quantum machine learning</x:v>
       </x:c>
       <x:c r="B124" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C124" s="2" t="str">
-        <x:v>Journal of the ACM</x:v>
+        <x:v>Quantum Science and Technology</x:v>
       </x:c>
       <x:c r="D124" s="2" t="str">
-        <x:v>Nai-Hui Chia, András Pal Gilyén, Tongyang Li, Han-Hsuan Lin, Ewin Tang, Chunhao WangAuthors Info &amp; Claims</x:v>
+        <x:v>James Dborin, Fergus Barratt, Vinul Wimalaweera, Lewis Wright and Andrew G Green</x:v>
       </x:c>
       <x:c r="E124" s="2" t="str">
-        <x:v>https://dl.acm.org/doi/abs/10.1145/3549524</x:v>
+        <x:v>https://iopscience.iop.org/article/10.1088/2058-9565/ac7073/meta</x:v>
       </x:c>
       <x:c r="F124" s="2" t="str">
         <x:v>QML</x:v>
@@ -3021,19 +3021,19 @@
     </x:row>
     <x:row r="125">
       <x:c r="A125" s="2" t="str">
-        <x:v>Verifying Fairness in Quantum Machine Learning (Book)</x:v>
+        <x:v>An orbital-based representation for accurate quantum machine learning </x:v>
       </x:c>
       <x:c r="B125" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C125" s="2" t="str">
-        <x:v>Computer Aided Verification</x:v>
+        <x:v>The Journal of Chemical Physics</x:v>
       </x:c>
       <x:c r="D125" s="2" t="str">
-        <x:v>Ji Guan, Wang Fang &amp; Mingsheng Ying   </x:v>
+        <x:v>Konstantin Karandashev; O. Anatole von Lilienfeld</x:v>
       </x:c>
       <x:c r="E125" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-13188-2_20</x:v>
+        <x:v>https://pubs.aip.org/aip/jcp/article-abstract/156/11/114101/2840879/An-orbital-based-representation-for-accurate?redirectedFrom=fulltext</x:v>
       </x:c>
       <x:c r="F125" s="2" t="str">
         <x:v>QML</x:v>
@@ -3041,19 +3041,19 @@
     </x:row>
     <x:row r="126">
       <x:c r="A126" s="2" t="str">
-        <x:v>Quantum Machine Learning in Drug Discovery: Current State and Challenges</x:v>
+        <x:v>Quantum Machine Learning Approach for Studying Atmospheric Cluster Formation</x:v>
       </x:c>
       <x:c r="B126" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C126" s="2" t="str">
-        <x:v>PCI '22: Proceedings of the 26th Pan-Hellenic Conference on Informatics</x:v>
+        <x:v>Environmental Science &amp; Technology Letters</x:v>
       </x:c>
       <x:c r="D126" s="2" t="str">
-        <x:v>Maria Avramouli, Ilias Savvas, Anna Vasilaki, Georgia Garani, Apostolos Xenakis &amp; Claims</x:v>
+        <x:v>Jakub Kubečka, Anders S. Christensen, Freja Rydahl Rasmussen,, Jonas Elm</x:v>
       </x:c>
       <x:c r="E126" s="2" t="str">
-        <x:v>https://dl.acm.org/doi/abs/10.1145/3575879.3576024</x:v>
+        <x:v>https://pubs.acs.org/doi/abs/10.1021/acs.estlett.1c00997</x:v>
       </x:c>
       <x:c r="F126" s="2" t="str">
         <x:v>QML</x:v>
@@ -3061,19 +3061,19 @@
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="2" t="str">
-        <x:v>A Preprocessing Perspective for Quantum Machine Learning Classification Advantage in Finance Using NISQ Algorithms</x:v>
+        <x:v>Overfitting in quantum machine learning and entangling dropout</x:v>
       </x:c>
       <x:c r="B127" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C127" s="2" t="str">
-        <x:v>Quantum Machine Learning 2022</x:v>
+        <x:v>Quantum Machine Intelligence</x:v>
       </x:c>
       <x:c r="D127" s="2" t="str">
-        <x:v>Javier Mancilla and Christophe Pere</x:v>
+        <x:v>Masahiro Kobayashi, Kouhei Nakaji &amp; Naoki Yamamoto</x:v>
       </x:c>
       <x:c r="E127" s="2" t="str">
-        <x:v>https://www.mdpi.com/1099-4300/24/11/1656</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s42484-022-00087-9</x:v>
       </x:c>
       <x:c r="F127" s="2" t="str">
         <x:v>QML</x:v>
@@ -3081,19 +3081,19 @@
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="2" t="str">
-        <x:v>Unsupervised quantum machine learning for fraud detection</x:v>
+        <x:v>Sampling-based Sublinear Low-rank Matrix Arithmetic Framework for Dequantizing Quantum Machine Learning</x:v>
       </x:c>
       <x:c r="B128" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C128" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Journal of the ACM</x:v>
       </x:c>
       <x:c r="D128" s="2" t="str">
-        <x:v>Oleksandr Kyriienko, Einar B. Magnusson</x:v>
+        <x:v>Nai-Hui Chia, András Pal Gilyén, Tongyang Li, Han-Hsuan Lin, Ewin Tang, Chunhao WangAuthors Info &amp; Claims</x:v>
       </x:c>
       <x:c r="E128" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2208.01203</x:v>
+        <x:v>https://dl.acm.org/doi/abs/10.1145/3549524</x:v>
       </x:c>
       <x:c r="F128" s="2" t="str">
         <x:v>QML</x:v>
@@ -3101,19 +3101,19 @@
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="2" t="str">
-        <x:v>Study of Feature Importance for Quantum Machine Learning Models</x:v>
+        <x:v>Verifying Fairness in Quantum Machine Learning (Book)</x:v>
       </x:c>
       <x:c r="B129" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C129" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Computer Aided Verification</x:v>
       </x:c>
       <x:c r="D129" s="2" t="str">
-        <x:v>Aaron Baughman, Kavitha Yogaraj, Raja Hebbar, Sudeep Ghosh, Rukhsan Ul Haq, Yoshika Chhabra</x:v>
+        <x:v>Ji Guan, Wang Fang &amp; Mingsheng Ying   </x:v>
       </x:c>
       <x:c r="E129" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2202.11204</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-13188-2_20</x:v>
       </x:c>
       <x:c r="F129" s="2" t="str">
         <x:v>QML</x:v>
@@ -3121,69 +3121,149 @@
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="2" t="str">
+        <x:v>Quantum Machine Learning in Drug Discovery: Current State and Challenges</x:v>
+      </x:c>
+      <x:c r="B130" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C130" s="2" t="str">
+        <x:v>PCI '22: Proceedings of the 26th Pan-Hellenic Conference on Informatics</x:v>
+      </x:c>
+      <x:c r="D130" s="2" t="str">
+        <x:v>Maria Avramouli, Ilias Savvas, Anna Vasilaki, Georgia Garani, Apostolos Xenakis &amp; Claims</x:v>
+      </x:c>
+      <x:c r="E130" s="2" t="str">
+        <x:v>https://dl.acm.org/doi/abs/10.1145/3575879.3576024</x:v>
+      </x:c>
+      <x:c r="F130" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="2" t="str">
+        <x:v>A Preprocessing Perspective for Quantum Machine Learning Classification Advantage in Finance Using NISQ Algorithms</x:v>
+      </x:c>
+      <x:c r="B131" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C131" s="2" t="str">
+        <x:v>Quantum Machine Learning 2022</x:v>
+      </x:c>
+      <x:c r="D131" s="2" t="str">
+        <x:v>Javier Mancilla and Christophe Pere</x:v>
+      </x:c>
+      <x:c r="E131" s="2" t="str">
+        <x:v>https://www.mdpi.com/1099-4300/24/11/1656</x:v>
+      </x:c>
+      <x:c r="F131" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="2" t="str">
+        <x:v>Unsupervised quantum machine learning for fraud detection</x:v>
+      </x:c>
+      <x:c r="B132" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C132" s="2" t="str">
+        <x:v>arxiv</x:v>
+      </x:c>
+      <x:c r="D132" s="2" t="str">
+        <x:v>Oleksandr Kyriienko, Einar B. Magnusson</x:v>
+      </x:c>
+      <x:c r="E132" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2208.01203</x:v>
+      </x:c>
+      <x:c r="F132" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="2" t="str">
+        <x:v>Study of Feature Importance for Quantum Machine Learning Models</x:v>
+      </x:c>
+      <x:c r="B133" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C133" s="2" t="str">
+        <x:v>arxiv</x:v>
+      </x:c>
+      <x:c r="D133" s="2" t="str">
+        <x:v>Aaron Baughman, Kavitha Yogaraj, Raja Hebbar, Sudeep Ghosh, Rukhsan Ul Haq, Yoshika Chhabra</x:v>
+      </x:c>
+      <x:c r="E133" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2202.11204</x:v>
+      </x:c>
+      <x:c r="F133" s="2" t="str">
+        <x:v>QML</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="2" t="str">
         <x:v>Noise-Resilient Quantum Machine Learning for Stability Assessment of Power Systems</x:v>
       </x:c>
-      <x:c r="B130" s="2" t="n">
-        <x:v>2022</x:v>
-      </x:c>
-      <x:c r="C130" s="2" t="str">
+      <x:c r="B134" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C134" s="2" t="str">
         <x:v>IEEE Transactions on Power Systems</x:v>
       </x:c>
-      <x:c r="D130" s="2" t="str">
+      <x:c r="D134" s="2" t="str">
         <x:v>Yifan Zhou; Peng Zhang</x:v>
       </x:c>
-      <x:c r="E130" s="2" t="str">
+      <x:c r="E134" s="2" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/9737359</x:v>
       </x:c>
-      <x:c r="F130" s="2" t="str">
+      <x:c r="F134" s="2" t="str">
         <x:v>QML</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="R5ba8f39f78df486c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="R53d346a45ff748af"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="Rae21786518e34ac0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="R8165f413b84d40af"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="R8ee1317757d84c2f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="R115271827bf84d48"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="Rb106ace84ed94ef1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R66331d08fbc840c1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="R45470fafa86b48f0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="Reb17a90abc114ed3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="Rfe7c7c7eea684ed4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="R3687ed7c4e7c4e1e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="Rc54f7845d8e74031"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="R406e07449b284419"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="R9fb60d5518874c46"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="Rd1a8621135144977"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="Rf53a0b17e32446b6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="Rb46faf76f7364355"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R8d4a733aebad464e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="Rb338bff052484588"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="Rac27338eac114fbc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R7039fd902a7f4062"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="R5ecadcbdc1c14dd2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="R656b1855a2b24d19"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="R6fe201a6e3d742f9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="R968187af881441ee"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="R8a5e9037e1124cac"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="Rf2f1df5b276a42b0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="Rbff2966486c5482b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="Rbb455fba97f94761"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="Re2a5312cdbe745cc"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="Rd6231e0cd9c542cb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="R917d35b4f92a4737"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="Rc14d852e8570442d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="R34be622369fc4963"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="Rc6231694bc99497f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="R7e0d9fccaccd46a9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="R90d892c9624546e5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="Red87a6fd61434a08"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="R63e515fb59a54d29"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="Ra9d3b159c786401f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="R208b4c7abddc4399"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="Red913564f59e483c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="Rc87e112048854e60"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="R7f8f86c97f0e4546"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="R45f79c11c323405a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="Rde4d1831beea4db6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="Rc59eece8bf334ef7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="Re0bb475c4d9a4239"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="R621cbc61789e4cd1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="R2988f3e19a484790"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="R9a344ffa86b846cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="R82f9ca34ad564726"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R66d63f7b42974989"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="R2812b1baa8384115"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="Ra8de5c2a8e9b41a8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="R17d0cd271b43440b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="R0c40520f73ee4d8a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R084e362a71b04aae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R55a67f88ff514276"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="R63441542cb6e4c0b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="R95563e72fa0d44ef"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R216b49b048b3432c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="R8deac321d78a4eae"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="R2744c6700df94616"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="R682b887022bb4a7e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="Rb0b0f218ebae4462"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="R45d3402e2e3c4bca"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="Rded624ca27a6472e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="R4148ef695e9b49ab"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="Rd5d87a034ba0476a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="R019e23a985724387"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="R895364dea62240b7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="Ra67b12d17a544a25"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="R824f17a37db5459f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="R699d632c98c04dea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="Rb23e48fe9f574809"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="Re61c6620b47046e7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="R6aa028a021b64ac5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="R300f7e3f81c341de"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="Rcadec0b2c5f6444c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="Rabb9485cb20241ae"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14459b1b52434b93"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23e295633bec4064"/>
 </x:worksheet>
 </file>
</xml_diff>